<commit_message>
Remove Zechen and rebalance to 3 reviewers
</commit_message>
<xml_diff>
--- a/ATTIS abstract submission_April 21, 2026_09.24_with_review_assignments.xlsx
+++ b/ATTIS abstract submission_April 21, 2026_09.24_with_review_assignments.xlsx
@@ -2153,7 +2153,7 @@
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>Garmire, Lana</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="F2" s="14" t="n"/>
@@ -2162,7 +2162,7 @@
       <c r="I2" s="14" t="n"/>
       <c r="J2" s="14" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="K2" s="14" t="n"/>
@@ -2171,27 +2171,19 @@
       <c r="N2" s="14" t="n"/>
       <c r="O2" s="14" t="inlineStr">
         <is>
-          <t>Mosa, Abu S</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="P2" s="14" t="n"/>
       <c r="Q2" s="14" t="n"/>
       <c r="R2" s="14" t="n"/>
       <c r="S2" s="14" t="n"/>
-      <c r="T2" s="14" t="inlineStr">
-        <is>
-          <t>Osborne, John D</t>
-        </is>
-      </c>
+      <c r="T2" s="14" t="n"/>
       <c r="U2" s="14" t="n"/>
       <c r="V2" s="14" t="n"/>
       <c r="W2" s="14" t="n"/>
       <c r="X2" s="14" t="n"/>
-      <c r="Y2" s="14" t="inlineStr">
-        <is>
-          <t>Amy Wang</t>
-        </is>
-      </c>
+      <c r="Y2" s="14" t="n"/>
       <c r="Z2" s="14" t="n"/>
       <c r="AA2" s="14" t="n"/>
       <c r="AB2" s="14" t="n"/>
@@ -2216,7 +2208,7 @@
       </c>
       <c r="E3" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="F3" s="14" t="n"/>
@@ -2225,7 +2217,7 @@
       <c r="I3" s="14" t="n"/>
       <c r="J3" s="14" t="inlineStr">
         <is>
-          <t>Garmire, Lana</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="K3" s="14" t="n"/>
@@ -2234,27 +2226,19 @@
       <c r="N3" s="14" t="n"/>
       <c r="O3" s="14" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Osborne, John D</t>
         </is>
       </c>
       <c r="P3" s="14" t="n"/>
       <c r="Q3" s="14" t="n"/>
       <c r="R3" s="14" t="n"/>
       <c r="S3" s="14" t="n"/>
-      <c r="T3" s="14" t="inlineStr">
-        <is>
-          <t>Mosa, Abu S</t>
-        </is>
-      </c>
+      <c r="T3" s="14" t="n"/>
       <c r="U3" s="14" t="n"/>
       <c r="V3" s="14" t="n"/>
       <c r="W3" s="14" t="n"/>
       <c r="X3" s="14" t="n"/>
-      <c r="Y3" s="14" t="inlineStr">
-        <is>
-          <t>Osborne, John D</t>
-        </is>
-      </c>
+      <c r="Y3" s="14" t="n"/>
       <c r="Z3" s="14" t="n"/>
       <c r="AA3" s="14" t="n"/>
       <c r="AB3" s="14" t="n"/>
@@ -2293,27 +2277,19 @@
       <c r="N4" s="14" t="n"/>
       <c r="O4" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Garmire, Lana</t>
         </is>
       </c>
       <c r="P4" s="14" t="n"/>
       <c r="Q4" s="14" t="n"/>
       <c r="R4" s="14" t="n"/>
       <c r="S4" s="14" t="n"/>
-      <c r="T4" s="14" t="inlineStr">
-        <is>
-          <t>Garmire, Lana</t>
-        </is>
-      </c>
+      <c r="T4" s="14" t="n"/>
       <c r="U4" s="14" t="n"/>
       <c r="V4" s="14" t="n"/>
       <c r="W4" s="14" t="n"/>
       <c r="X4" s="14" t="n"/>
-      <c r="Y4" s="14" t="inlineStr">
-        <is>
-          <t>Jinzhuang Dou</t>
-        </is>
-      </c>
+      <c r="Y4" s="14" t="n"/>
       <c r="Z4" s="14" t="n"/>
       <c r="AA4" s="14" t="n"/>
       <c r="AB4" s="14" t="n"/>
@@ -2338,7 +2314,7 @@
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
-          <t>Osborne, John D</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="F5" s="14" t="n"/>
@@ -2347,7 +2323,7 @@
       <c r="I5" s="14" t="n"/>
       <c r="J5" s="14" t="inlineStr">
         <is>
-          <t>Amy Wang</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="K5" s="14" t="n"/>
@@ -2356,27 +2332,19 @@
       <c r="N5" s="14" t="n"/>
       <c r="O5" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="P5" s="14" t="n"/>
       <c r="Q5" s="14" t="n"/>
       <c r="R5" s="14" t="n"/>
       <c r="S5" s="14" t="n"/>
-      <c r="T5" s="14" t="inlineStr">
-        <is>
-          <t>Chen, Jin (Campus)</t>
-        </is>
-      </c>
+      <c r="T5" s="14" t="n"/>
       <c r="U5" s="14" t="n"/>
       <c r="V5" s="14" t="n"/>
       <c r="W5" s="14" t="n"/>
       <c r="X5" s="14" t="n"/>
-      <c r="Y5" s="14" t="inlineStr">
-        <is>
-          <t>Chong, Zechen</t>
-        </is>
-      </c>
+      <c r="Y5" s="14" t="n"/>
       <c r="Z5" s="14" t="n"/>
       <c r="AA5" s="14" t="n"/>
       <c r="AB5" s="14" t="n"/>
@@ -2401,7 +2369,7 @@
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="F6" s="14" t="n"/>
@@ -2410,7 +2378,7 @@
       <c r="I6" s="14" t="n"/>
       <c r="J6" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jin (Campus)</t>
+          <t>Osborne, John D</t>
         </is>
       </c>
       <c r="K6" s="14" t="n"/>
@@ -2419,27 +2387,19 @@
       <c r="N6" s="14" t="n"/>
       <c r="O6" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="P6" s="14" t="n"/>
       <c r="Q6" s="14" t="n"/>
       <c r="R6" s="14" t="n"/>
       <c r="S6" s="14" t="n"/>
-      <c r="T6" s="14" t="inlineStr">
-        <is>
-          <t>Jinzhuang Dou</t>
-        </is>
-      </c>
+      <c r="T6" s="14" t="n"/>
       <c r="U6" s="14" t="n"/>
       <c r="V6" s="14" t="n"/>
       <c r="W6" s="14" t="n"/>
       <c r="X6" s="14" t="n"/>
-      <c r="Y6" s="14" t="inlineStr">
-        <is>
-          <t>Mosa, Abu S</t>
-        </is>
-      </c>
+      <c r="Y6" s="14" t="n"/>
       <c r="Z6" s="14" t="n"/>
       <c r="AA6" s="14" t="n"/>
       <c r="AB6" s="14" t="n"/>
@@ -2464,7 +2424,7 @@
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="F7" s="14" t="n"/>
@@ -2473,7 +2433,7 @@
       <c r="I7" s="14" t="n"/>
       <c r="J7" s="14" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="K7" s="14" t="n"/>
@@ -2482,27 +2442,19 @@
       <c r="N7" s="14" t="n"/>
       <c r="O7" s="14" t="inlineStr">
         <is>
-          <t>Mosa, Abu S</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="P7" s="14" t="n"/>
       <c r="Q7" s="14" t="n"/>
       <c r="R7" s="14" t="n"/>
       <c r="S7" s="14" t="n"/>
-      <c r="T7" s="14" t="inlineStr">
-        <is>
-          <t>Osborne, John D</t>
-        </is>
-      </c>
+      <c r="T7" s="14" t="n"/>
       <c r="U7" s="14" t="n"/>
       <c r="V7" s="14" t="n"/>
       <c r="W7" s="14" t="n"/>
       <c r="X7" s="14" t="n"/>
-      <c r="Y7" s="14" t="inlineStr">
-        <is>
-          <t>Amy Wang</t>
-        </is>
-      </c>
+      <c r="Y7" s="14" t="n"/>
       <c r="Z7" s="14" t="n"/>
       <c r="AA7" s="14" t="n"/>
       <c r="AB7" s="14" t="n"/>
@@ -2552,20 +2504,12 @@
       <c r="Q8" s="14" t="n"/>
       <c r="R8" s="14" t="n"/>
       <c r="S8" s="14" t="n"/>
-      <c r="T8" s="14" t="inlineStr">
-        <is>
-          <t>Chen, Jake Y</t>
-        </is>
-      </c>
+      <c r="T8" s="14" t="n"/>
       <c r="U8" s="14" t="n"/>
       <c r="V8" s="14" t="n"/>
       <c r="W8" s="14" t="n"/>
       <c r="X8" s="14" t="n"/>
-      <c r="Y8" s="14" t="inlineStr">
-        <is>
-          <t>Chen, Jin (Campus)</t>
-        </is>
-      </c>
+      <c r="Y8" s="14" t="n"/>
       <c r="Z8" s="14" t="n"/>
       <c r="AA8" s="14" t="n"/>
       <c r="AB8" s="14" t="n"/>
@@ -2590,7 +2534,7 @@
       </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="F9" s="14" t="n"/>
@@ -2599,7 +2543,7 @@
       <c r="I9" s="14" t="n"/>
       <c r="J9" s="14" t="inlineStr">
         <is>
-          <t>Garmire, Lana</t>
+          <t>Osborne, John D</t>
         </is>
       </c>
       <c r="K9" s="14" t="n"/>
@@ -2608,27 +2552,19 @@
       <c r="N9" s="14" t="n"/>
       <c r="O9" s="14" t="inlineStr">
         <is>
-          <t>Mosa, Abu S</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="P9" s="14" t="n"/>
       <c r="Q9" s="14" t="n"/>
       <c r="R9" s="14" t="n"/>
       <c r="S9" s="14" t="n"/>
-      <c r="T9" s="14" t="inlineStr">
-        <is>
-          <t>Osborne, John D</t>
-        </is>
-      </c>
+      <c r="T9" s="14" t="n"/>
       <c r="U9" s="14" t="n"/>
       <c r="V9" s="14" t="n"/>
       <c r="W9" s="14" t="n"/>
       <c r="X9" s="14" t="n"/>
-      <c r="Y9" s="14" t="inlineStr">
-        <is>
-          <t>Amy Wang</t>
-        </is>
-      </c>
+      <c r="Y9" s="14" t="n"/>
       <c r="Z9" s="14" t="n"/>
       <c r="AA9" s="14" t="n"/>
       <c r="AB9" s="14" t="n"/>
@@ -2653,7 +2589,7 @@
       </c>
       <c r="E10" s="14" t="inlineStr">
         <is>
-          <t>Amy Wang</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="F10" s="14" t="n"/>
@@ -2662,7 +2598,7 @@
       <c r="I10" s="14" t="n"/>
       <c r="J10" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="K10" s="14" t="n"/>
@@ -2671,27 +2607,19 @@
       <c r="N10" s="14" t="n"/>
       <c r="O10" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jin (Campus)</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="P10" s="14" t="n"/>
       <c r="Q10" s="14" t="n"/>
       <c r="R10" s="14" t="n"/>
       <c r="S10" s="14" t="n"/>
-      <c r="T10" s="14" t="inlineStr">
-        <is>
-          <t>Chong, Zechen</t>
-        </is>
-      </c>
+      <c r="T10" s="14" t="n"/>
       <c r="U10" s="14" t="n"/>
       <c r="V10" s="14" t="n"/>
       <c r="W10" s="14" t="n"/>
       <c r="X10" s="14" t="n"/>
-      <c r="Y10" s="14" t="inlineStr">
-        <is>
-          <t>Jinzhuang Dou</t>
-        </is>
-      </c>
+      <c r="Y10" s="14" t="n"/>
       <c r="Z10" s="14" t="n"/>
       <c r="AA10" s="14" t="n"/>
       <c r="AB10" s="14" t="n"/>
@@ -2716,7 +2644,7 @@
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="F11" s="14" t="n"/>
@@ -2725,7 +2653,7 @@
       <c r="I11" s="14" t="n"/>
       <c r="J11" s="14" t="inlineStr">
         <is>
-          <t>Amy Wang</t>
+          <t>Osborne, John D</t>
         </is>
       </c>
       <c r="K11" s="14" t="n"/>
@@ -2734,27 +2662,19 @@
       <c r="N11" s="14" t="n"/>
       <c r="O11" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jin (Campus)</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="P11" s="14" t="n"/>
       <c r="Q11" s="14" t="n"/>
       <c r="R11" s="14" t="n"/>
       <c r="S11" s="14" t="n"/>
-      <c r="T11" s="14" t="inlineStr">
-        <is>
-          <t>Chong, Zechen</t>
-        </is>
-      </c>
+      <c r="T11" s="14" t="n"/>
       <c r="U11" s="14" t="n"/>
       <c r="V11" s="14" t="n"/>
       <c r="W11" s="14" t="n"/>
       <c r="X11" s="14" t="n"/>
-      <c r="Y11" s="14" t="inlineStr">
-        <is>
-          <t>Jinzhuang Dou</t>
-        </is>
-      </c>
+      <c r="Y11" s="14" t="n"/>
       <c r="Z11" s="14" t="n"/>
       <c r="AA11" s="14" t="n"/>
       <c r="AB11" s="14" t="n"/>
@@ -2775,7 +2695,7 @@
       </c>
       <c r="E12" s="14" t="inlineStr">
         <is>
-          <t>Osborne, John D</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="F12" s="14" t="n"/>
@@ -2784,7 +2704,7 @@
       <c r="I12" s="14" t="n"/>
       <c r="J12" s="14" t="inlineStr">
         <is>
-          <t>Amy Wang</t>
+          <t>Garmire, Lana</t>
         </is>
       </c>
       <c r="K12" s="14" t="n"/>
@@ -2793,27 +2713,19 @@
       <c r="N12" s="14" t="n"/>
       <c r="O12" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="P12" s="14" t="n"/>
       <c r="Q12" s="14" t="n"/>
       <c r="R12" s="14" t="n"/>
       <c r="S12" s="14" t="n"/>
-      <c r="T12" s="14" t="inlineStr">
-        <is>
-          <t>Chen, Jin (Campus)</t>
-        </is>
-      </c>
+      <c r="T12" s="14" t="n"/>
       <c r="U12" s="14" t="n"/>
       <c r="V12" s="14" t="n"/>
       <c r="W12" s="14" t="n"/>
       <c r="X12" s="14" t="n"/>
-      <c r="Y12" s="14" t="inlineStr">
-        <is>
-          <t>Chong, Zechen</t>
-        </is>
-      </c>
+      <c r="Y12" s="14" t="n"/>
       <c r="Z12" s="14" t="n"/>
       <c r="AA12" s="14" t="n"/>
       <c r="AB12" s="14" t="n"/>
@@ -2838,7 +2750,7 @@
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jin (Campus)</t>
+          <t>Osborne, John D</t>
         </is>
       </c>
       <c r="F13" s="14" t="n"/>
@@ -2847,7 +2759,7 @@
       <c r="I13" s="14" t="n"/>
       <c r="J13" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="K13" s="14" t="n"/>
@@ -2856,27 +2768,19 @@
       <c r="N13" s="14" t="n"/>
       <c r="O13" s="14" t="inlineStr">
         <is>
-          <t>Garmire, Lana</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="P13" s="14" t="n"/>
       <c r="Q13" s="14" t="n"/>
       <c r="R13" s="14" t="n"/>
       <c r="S13" s="14" t="n"/>
-      <c r="T13" s="14" t="inlineStr">
-        <is>
-          <t>Jinzhuang Dou</t>
-        </is>
-      </c>
+      <c r="T13" s="14" t="n"/>
       <c r="U13" s="14" t="n"/>
       <c r="V13" s="14" t="n"/>
       <c r="W13" s="14" t="n"/>
       <c r="X13" s="14" t="n"/>
-      <c r="Y13" s="14" t="inlineStr">
-        <is>
-          <t>Mosa, Abu S</t>
-        </is>
-      </c>
+      <c r="Y13" s="14" t="n"/>
       <c r="Z13" s="14" t="n"/>
       <c r="AA13" s="14" t="n"/>
       <c r="AB13" s="14" t="n"/>
@@ -2901,7 +2805,7 @@
       </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Garmire, Lana</t>
         </is>
       </c>
       <c r="F14" s="14" t="n"/>
@@ -2910,7 +2814,7 @@
       <c r="I14" s="14" t="n"/>
       <c r="J14" s="14" t="inlineStr">
         <is>
-          <t>Mosa, Abu S</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="K14" s="14" t="n"/>
@@ -2919,27 +2823,19 @@
       <c r="N14" s="14" t="n"/>
       <c r="O14" s="14" t="inlineStr">
         <is>
-          <t>Osborne, John D</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="P14" s="14" t="n"/>
       <c r="Q14" s="14" t="n"/>
       <c r="R14" s="14" t="n"/>
       <c r="S14" s="14" t="n"/>
-      <c r="T14" s="14" t="inlineStr">
-        <is>
-          <t>Amy Wang</t>
-        </is>
-      </c>
+      <c r="T14" s="14" t="n"/>
       <c r="U14" s="14" t="n"/>
       <c r="V14" s="14" t="n"/>
       <c r="W14" s="14" t="n"/>
       <c r="X14" s="14" t="n"/>
-      <c r="Y14" s="14" t="inlineStr">
-        <is>
-          <t>Chen, Jake Y</t>
-        </is>
-      </c>
+      <c r="Y14" s="14" t="n"/>
       <c r="Z14" s="14" t="n"/>
       <c r="AA14" s="14" t="n"/>
       <c r="AB14" s="14" t="n"/>
@@ -2989,20 +2885,12 @@
       <c r="Q15" s="14" t="n"/>
       <c r="R15" s="14" t="n"/>
       <c r="S15" s="14" t="n"/>
-      <c r="T15" s="14" t="inlineStr">
-        <is>
-          <t>Mosa, Abu S</t>
-        </is>
-      </c>
+      <c r="T15" s="14" t="n"/>
       <c r="U15" s="14" t="n"/>
       <c r="V15" s="14" t="n"/>
       <c r="W15" s="14" t="n"/>
       <c r="X15" s="14" t="n"/>
-      <c r="Y15" s="14" t="inlineStr">
-        <is>
-          <t>Osborne, John D</t>
-        </is>
-      </c>
+      <c r="Y15" s="14" t="n"/>
       <c r="Z15" s="14" t="n"/>
       <c r="AA15" s="14" t="n"/>
       <c r="AB15" s="14" t="n"/>
@@ -3027,7 +2915,7 @@
       </c>
       <c r="E16" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="F16" s="14" t="n"/>
@@ -3036,7 +2924,7 @@
       <c r="I16" s="14" t="n"/>
       <c r="J16" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jin (Campus)</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="K16" s="14" t="n"/>
@@ -3045,27 +2933,19 @@
       <c r="N16" s="14" t="n"/>
       <c r="O16" s="14" t="inlineStr">
         <is>
-          <t>Osborne, John D</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="P16" s="14" t="n"/>
       <c r="Q16" s="14" t="n"/>
       <c r="R16" s="14" t="n"/>
       <c r="S16" s="14" t="n"/>
-      <c r="T16" s="14" t="inlineStr">
-        <is>
-          <t>Amy Wang</t>
-        </is>
-      </c>
+      <c r="T16" s="14" t="n"/>
       <c r="U16" s="14" t="n"/>
       <c r="V16" s="14" t="n"/>
       <c r="W16" s="14" t="n"/>
       <c r="X16" s="14" t="n"/>
-      <c r="Y16" s="14" t="inlineStr">
-        <is>
-          <t>Chong, Zechen</t>
-        </is>
-      </c>
+      <c r="Y16" s="14" t="n"/>
       <c r="Z16" s="14" t="n"/>
       <c r="AA16" s="14" t="n"/>
       <c r="AB16" s="14" t="n"/>
@@ -3115,20 +2995,12 @@
       <c r="Q17" s="14" t="n"/>
       <c r="R17" s="14" t="n"/>
       <c r="S17" s="14" t="n"/>
-      <c r="T17" s="14" t="inlineStr">
-        <is>
-          <t>Chong, Zechen</t>
-        </is>
-      </c>
+      <c r="T17" s="14" t="n"/>
       <c r="U17" s="14" t="n"/>
       <c r="V17" s="14" t="n"/>
       <c r="W17" s="14" t="n"/>
       <c r="X17" s="14" t="n"/>
-      <c r="Y17" s="14" t="inlineStr">
-        <is>
-          <t>Garmire, Lana</t>
-        </is>
-      </c>
+      <c r="Y17" s="14" t="n"/>
       <c r="Z17" s="14" t="n"/>
       <c r="AA17" s="14" t="n"/>
       <c r="AB17" s="14" t="n"/>
@@ -3162,7 +3034,7 @@
       <c r="I18" s="14" t="n"/>
       <c r="J18" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="K18" s="14" t="n"/>
@@ -3171,27 +3043,19 @@
       <c r="N18" s="14" t="n"/>
       <c r="O18" s="14" t="inlineStr">
         <is>
-          <t>Garmire, Lana</t>
+          <t>Osborne, John D</t>
         </is>
       </c>
       <c r="P18" s="14" t="n"/>
       <c r="Q18" s="14" t="n"/>
       <c r="R18" s="14" t="n"/>
       <c r="S18" s="14" t="n"/>
-      <c r="T18" s="14" t="inlineStr">
-        <is>
-          <t>Jinzhuang Dou</t>
-        </is>
-      </c>
+      <c r="T18" s="14" t="n"/>
       <c r="U18" s="14" t="n"/>
       <c r="V18" s="14" t="n"/>
       <c r="W18" s="14" t="n"/>
       <c r="X18" s="14" t="n"/>
-      <c r="Y18" s="14" t="inlineStr">
-        <is>
-          <t>Mosa, Abu S</t>
-        </is>
-      </c>
+      <c r="Y18" s="14" t="n"/>
       <c r="Z18" s="14" t="n"/>
       <c r="AA18" s="14" t="n"/>
       <c r="AB18" s="14" t="n"/>
@@ -3234,27 +3098,19 @@
       <c r="N19" s="14" t="n"/>
       <c r="O19" s="14" t="inlineStr">
         <is>
-          <t>Mosa, Abu S</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="P19" s="14" t="n"/>
       <c r="Q19" s="14" t="n"/>
       <c r="R19" s="14" t="n"/>
       <c r="S19" s="14" t="n"/>
-      <c r="T19" s="14" t="inlineStr">
-        <is>
-          <t>Osborne, John D</t>
-        </is>
-      </c>
+      <c r="T19" s="14" t="n"/>
       <c r="U19" s="14" t="n"/>
       <c r="V19" s="14" t="n"/>
       <c r="W19" s="14" t="n"/>
       <c r="X19" s="14" t="n"/>
-      <c r="Y19" s="14" t="inlineStr">
-        <is>
-          <t>Amy Wang</t>
-        </is>
-      </c>
+      <c r="Y19" s="14" t="n"/>
       <c r="Z19" s="14" t="n"/>
       <c r="AA19" s="14" t="n"/>
       <c r="AB19" s="14" t="n"/>
@@ -3288,7 +3144,7 @@
       <c r="I20" s="14" t="n"/>
       <c r="J20" s="14" t="inlineStr">
         <is>
-          <t>Amy Wang</t>
+          <t>Osborne, John D</t>
         </is>
       </c>
       <c r="K20" s="14" t="n"/>
@@ -3297,27 +3153,19 @@
       <c r="N20" s="14" t="n"/>
       <c r="O20" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jin (Campus)</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="P20" s="14" t="n"/>
       <c r="Q20" s="14" t="n"/>
       <c r="R20" s="14" t="n"/>
       <c r="S20" s="14" t="n"/>
-      <c r="T20" s="14" t="inlineStr">
-        <is>
-          <t>Chong, Zechen</t>
-        </is>
-      </c>
+      <c r="T20" s="14" t="n"/>
       <c r="U20" s="14" t="n"/>
       <c r="V20" s="14" t="n"/>
       <c r="W20" s="14" t="n"/>
       <c r="X20" s="14" t="n"/>
-      <c r="Y20" s="14" t="inlineStr">
-        <is>
-          <t>Jinzhuang Dou</t>
-        </is>
-      </c>
+      <c r="Y20" s="14" t="n"/>
       <c r="Z20" s="14" t="n"/>
       <c r="AA20" s="14" t="n"/>
       <c r="AB20" s="14" t="n"/>
@@ -3342,7 +3190,7 @@
       </c>
       <c r="E21" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Garmire, Lana</t>
         </is>
       </c>
       <c r="F21" s="14" t="n"/>
@@ -3351,7 +3199,7 @@
       <c r="I21" s="14" t="n"/>
       <c r="J21" s="14" t="inlineStr">
         <is>
-          <t>Garmire, Lana</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="K21" s="14" t="n"/>
@@ -3360,27 +3208,19 @@
       <c r="N21" s="14" t="n"/>
       <c r="O21" s="14" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="P21" s="14" t="n"/>
       <c r="Q21" s="14" t="n"/>
       <c r="R21" s="14" t="n"/>
       <c r="S21" s="14" t="n"/>
-      <c r="T21" s="14" t="inlineStr">
-        <is>
-          <t>Mosa, Abu S</t>
-        </is>
-      </c>
+      <c r="T21" s="14" t="n"/>
       <c r="U21" s="14" t="n"/>
       <c r="V21" s="14" t="n"/>
       <c r="W21" s="14" t="n"/>
       <c r="X21" s="14" t="n"/>
-      <c r="Y21" s="14" t="inlineStr">
-        <is>
-          <t>Osborne, John D</t>
-        </is>
-      </c>
+      <c r="Y21" s="14" t="n"/>
       <c r="Z21" s="14" t="n"/>
       <c r="AA21" s="14" t="n"/>
       <c r="AB21" s="14" t="n"/>
@@ -3405,7 +3245,7 @@
       </c>
       <c r="E22" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Osborne, John D</t>
         </is>
       </c>
       <c r="F22" s="14" t="n"/>
@@ -3414,7 +3254,7 @@
       <c r="I22" s="14" t="n"/>
       <c r="J22" s="14" t="inlineStr">
         <is>
-          <t>Garmire, Lana</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="K22" s="14" t="n"/>
@@ -3423,27 +3263,19 @@
       <c r="N22" s="14" t="n"/>
       <c r="O22" s="14" t="inlineStr">
         <is>
-          <t>Osborne, John D</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="P22" s="14" t="n"/>
       <c r="Q22" s="14" t="n"/>
       <c r="R22" s="14" t="n"/>
       <c r="S22" s="14" t="n"/>
-      <c r="T22" s="14" t="inlineStr">
-        <is>
-          <t>Amy Wang</t>
-        </is>
-      </c>
+      <c r="T22" s="14" t="n"/>
       <c r="U22" s="14" t="n"/>
       <c r="V22" s="14" t="n"/>
       <c r="W22" s="14" t="n"/>
       <c r="X22" s="14" t="n"/>
-      <c r="Y22" s="14" t="inlineStr">
-        <is>
-          <t>Chen, Jin (Campus)</t>
-        </is>
-      </c>
+      <c r="Y22" s="14" t="n"/>
       <c r="Z22" s="14" t="n"/>
       <c r="AA22" s="14" t="n"/>
       <c r="AB22" s="14" t="n"/>
@@ -3468,7 +3300,7 @@
       </c>
       <c r="E23" s="14" t="inlineStr">
         <is>
-          <t>Mosa, Abu S</t>
+          <t>Garmire, Lana</t>
         </is>
       </c>
       <c r="F23" s="14" t="n"/>
@@ -3477,7 +3309,7 @@
       <c r="I23" s="14" t="n"/>
       <c r="J23" s="14" t="inlineStr">
         <is>
-          <t>Osborne, John D</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="K23" s="14" t="n"/>
@@ -3486,27 +3318,19 @@
       <c r="N23" s="14" t="n"/>
       <c r="O23" s="14" t="inlineStr">
         <is>
-          <t>Amy Wang</t>
+          <t>Osborne, John D</t>
         </is>
       </c>
       <c r="P23" s="14" t="n"/>
       <c r="Q23" s="14" t="n"/>
       <c r="R23" s="14" t="n"/>
       <c r="S23" s="14" t="n"/>
-      <c r="T23" s="14" t="inlineStr">
-        <is>
-          <t>Chen, Jake Y</t>
-        </is>
-      </c>
+      <c r="T23" s="14" t="n"/>
       <c r="U23" s="14" t="n"/>
       <c r="V23" s="14" t="n"/>
       <c r="W23" s="14" t="n"/>
       <c r="X23" s="14" t="n"/>
-      <c r="Y23" s="14" t="inlineStr">
-        <is>
-          <t>Chen, Jin (Campus)</t>
-        </is>
-      </c>
+      <c r="Y23" s="14" t="n"/>
       <c r="Z23" s="14" t="n"/>
       <c r="AA23" s="14" t="n"/>
       <c r="AB23" s="14" t="n"/>
@@ -3531,7 +3355,7 @@
       </c>
       <c r="E24" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Garmire, Lana</t>
         </is>
       </c>
       <c r="F24" s="14" t="n"/>
@@ -3540,7 +3364,7 @@
       <c r="I24" s="14" t="n"/>
       <c r="J24" s="14" t="inlineStr">
         <is>
-          <t>Garmire, Lana</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="K24" s="14" t="n"/>
@@ -3549,27 +3373,19 @@
       <c r="N24" s="14" t="n"/>
       <c r="O24" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jin (Campus)</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="P24" s="14" t="n"/>
       <c r="Q24" s="14" t="n"/>
       <c r="R24" s="14" t="n"/>
       <c r="S24" s="14" t="n"/>
-      <c r="T24" s="14" t="inlineStr">
-        <is>
-          <t>Jinzhuang Dou</t>
-        </is>
-      </c>
+      <c r="T24" s="14" t="n"/>
       <c r="U24" s="14" t="n"/>
       <c r="V24" s="14" t="n"/>
       <c r="W24" s="14" t="n"/>
       <c r="X24" s="14" t="n"/>
-      <c r="Y24" s="14" t="inlineStr">
-        <is>
-          <t>Mosa, Abu S</t>
-        </is>
-      </c>
+      <c r="Y24" s="14" t="n"/>
       <c r="Z24" s="14" t="n"/>
       <c r="AA24" s="14" t="n"/>
       <c r="AB24" s="14" t="n"/>
@@ -3594,7 +3410,7 @@
       </c>
       <c r="E25" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Osborne, John D</t>
         </is>
       </c>
       <c r="F25" s="14" t="n"/>
@@ -3603,7 +3419,7 @@
       <c r="I25" s="14" t="n"/>
       <c r="J25" s="14" t="inlineStr">
         <is>
-          <t>Garmire, Lana</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="K25" s="14" t="n"/>
@@ -3612,27 +3428,19 @@
       <c r="N25" s="14" t="n"/>
       <c r="O25" s="14" t="inlineStr">
         <is>
-          <t>Mosa, Abu S</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="P25" s="14" t="n"/>
       <c r="Q25" s="14" t="n"/>
       <c r="R25" s="14" t="n"/>
       <c r="S25" s="14" t="n"/>
-      <c r="T25" s="14" t="inlineStr">
-        <is>
-          <t>Osborne, John D</t>
-        </is>
-      </c>
+      <c r="T25" s="14" t="n"/>
       <c r="U25" s="14" t="n"/>
       <c r="V25" s="14" t="n"/>
       <c r="W25" s="14" t="n"/>
       <c r="X25" s="14" t="n"/>
-      <c r="Y25" s="14" t="inlineStr">
-        <is>
-          <t>Amy Wang</t>
-        </is>
-      </c>
+      <c r="Y25" s="14" t="n"/>
       <c r="Z25" s="14" t="n"/>
       <c r="AA25" s="14" t="n"/>
       <c r="AB25" s="14" t="n"/>
@@ -3666,7 +3474,7 @@
       <c r="I26" s="14" t="n"/>
       <c r="J26" s="14" t="inlineStr">
         <is>
-          <t>Amy Wang</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="K26" s="14" t="n"/>
@@ -3675,27 +3483,19 @@
       <c r="N26" s="14" t="n"/>
       <c r="O26" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="P26" s="14" t="n"/>
       <c r="Q26" s="14" t="n"/>
       <c r="R26" s="14" t="n"/>
       <c r="S26" s="14" t="n"/>
-      <c r="T26" s="14" t="inlineStr">
-        <is>
-          <t>Chen, Jin (Campus)</t>
-        </is>
-      </c>
+      <c r="T26" s="14" t="n"/>
       <c r="U26" s="14" t="n"/>
       <c r="V26" s="14" t="n"/>
       <c r="W26" s="14" t="n"/>
       <c r="X26" s="14" t="n"/>
-      <c r="Y26" s="14" t="inlineStr">
-        <is>
-          <t>Jinzhuang Dou</t>
-        </is>
-      </c>
+      <c r="Y26" s="14" t="n"/>
       <c r="Z26" s="14" t="n"/>
       <c r="AA26" s="14" t="n"/>
       <c r="AB26" s="14" t="n"/>
@@ -3729,7 +3529,7 @@
       <c r="I27" s="14" t="n"/>
       <c r="J27" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jin (Campus)</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="K27" s="14" t="n"/>
@@ -3738,27 +3538,19 @@
       <c r="N27" s="14" t="n"/>
       <c r="O27" s="14" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="P27" s="14" t="n"/>
       <c r="Q27" s="14" t="n"/>
       <c r="R27" s="14" t="n"/>
       <c r="S27" s="14" t="n"/>
-      <c r="T27" s="14" t="inlineStr">
-        <is>
-          <t>Mosa, Abu S</t>
-        </is>
-      </c>
+      <c r="T27" s="14" t="n"/>
       <c r="U27" s="14" t="n"/>
       <c r="V27" s="14" t="n"/>
       <c r="W27" s="14" t="n"/>
       <c r="X27" s="14" t="n"/>
-      <c r="Y27" s="14" t="inlineStr">
-        <is>
-          <t>Osborne, John D</t>
-        </is>
-      </c>
+      <c r="Y27" s="14" t="n"/>
       <c r="Z27" s="14" t="n"/>
       <c r="AA27" s="14" t="n"/>
       <c r="AB27" s="14" t="n"/>
@@ -3792,7 +3584,7 @@
       <c r="I28" s="14" t="n"/>
       <c r="J28" s="14" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="K28" s="14" t="n"/>
@@ -3808,20 +3600,12 @@
       <c r="Q28" s="14" t="n"/>
       <c r="R28" s="14" t="n"/>
       <c r="S28" s="14" t="n"/>
-      <c r="T28" s="14" t="inlineStr">
-        <is>
-          <t>Amy Wang</t>
-        </is>
-      </c>
+      <c r="T28" s="14" t="n"/>
       <c r="U28" s="14" t="n"/>
       <c r="V28" s="14" t="n"/>
       <c r="W28" s="14" t="n"/>
       <c r="X28" s="14" t="n"/>
-      <c r="Y28" s="14" t="inlineStr">
-        <is>
-          <t>Chen, Jake Y</t>
-        </is>
-      </c>
+      <c r="Y28" s="14" t="n"/>
       <c r="Z28" s="14" t="n"/>
       <c r="AA28" s="14" t="n"/>
       <c r="AB28" s="14" t="n"/>
@@ -3864,27 +3648,19 @@
       <c r="N29" s="14" t="n"/>
       <c r="O29" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jin (Campus)</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="P29" s="14" t="n"/>
       <c r="Q29" s="14" t="n"/>
       <c r="R29" s="14" t="n"/>
       <c r="S29" s="14" t="n"/>
-      <c r="T29" s="14" t="inlineStr">
-        <is>
-          <t>Chong, Zechen</t>
-        </is>
-      </c>
+      <c r="T29" s="14" t="n"/>
       <c r="U29" s="14" t="n"/>
       <c r="V29" s="14" t="n"/>
       <c r="W29" s="14" t="n"/>
       <c r="X29" s="14" t="n"/>
-      <c r="Y29" s="14" t="inlineStr">
-        <is>
-          <t>Mosa, Abu S</t>
-        </is>
-      </c>
+      <c r="Y29" s="14" t="n"/>
       <c r="Z29" s="14" t="n"/>
       <c r="AA29" s="14" t="n"/>
       <c r="AB29" s="14" t="n"/>
@@ -3909,7 +3685,7 @@
       </c>
       <c r="E30" s="14" t="inlineStr">
         <is>
-          <t>Garmire, Lana</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="F30" s="14" t="n"/>
@@ -3918,7 +3694,7 @@
       <c r="I30" s="14" t="n"/>
       <c r="J30" s="14" t="inlineStr">
         <is>
-          <t>Mosa, Abu S</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="K30" s="14" t="n"/>
@@ -3927,27 +3703,19 @@
       <c r="N30" s="14" t="n"/>
       <c r="O30" s="14" t="inlineStr">
         <is>
-          <t>Osborne, John D</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="P30" s="14" t="n"/>
       <c r="Q30" s="14" t="n"/>
       <c r="R30" s="14" t="n"/>
       <c r="S30" s="14" t="n"/>
-      <c r="T30" s="14" t="inlineStr">
-        <is>
-          <t>Amy Wang</t>
-        </is>
-      </c>
+      <c r="T30" s="14" t="n"/>
       <c r="U30" s="14" t="n"/>
       <c r="V30" s="14" t="n"/>
       <c r="W30" s="14" t="n"/>
       <c r="X30" s="14" t="n"/>
-      <c r="Y30" s="14" t="inlineStr">
-        <is>
-          <t>Chen, Jake Y</t>
-        </is>
-      </c>
+      <c r="Y30" s="14" t="n"/>
       <c r="Z30" s="14" t="n"/>
       <c r="AA30" s="14" t="n"/>
       <c r="AB30" s="14" t="n"/>

</xml_diff>

<commit_message>
Update abstract workbook from April 21 submissions; add SCG to review grid
Merge Sheet0 from parent submission spreadsheet into assignments workbook.
Append Review_Assignments row for abstract 30 (SCG) with provisional reviewers.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/ATTIS abstract submission_April 21, 2026_09.24_with_review_assignments.xlsx
+++ b/ATTIS abstract submission_April 21, 2026_09.24_with_review_assignments.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="2120" yWindow="500" windowWidth="37020" windowHeight="21100" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet0" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Review_Assignments" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet0" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review_Assignments" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet0'!$B$1:$H$26</definedName>
@@ -820,7 +820,18 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Drug repurposing offers a scalable route to accelerate therapeutic discovery, yet existing approaches based on single-cell RNA sequencing (scRNA-seq) often overlook spatial tissue context, limiting their ability to capture microenvironment-dependent drug responses. Here we present STDrug, a spatially informed computational framework that integrates spatial transcriptomics, graph-based modeling, and multimodal learning to enable patient-specific therapeutic prioritization. STDrug identifies and aligns disease and control spatial domains using graph convolutional networks and coherent point drift, and prioritizes candidate drugs through an integrative scoring scheme combining tumor-reversible gene signatures, perturbation-based reversal scores, and knowledge-guided gene weighting within a machine learning framework. By modeling spatial domain interactions alongside predicted drug efficacy and toxicity, STDrug generates robust patient-level drug scores. Across hepatocellular carcinoma and prostate cancer datasets, STDrug outperforms existing single-cell and spatial transcriptomics–based drug repurposing methods, achieving signficantly improved predictive accuracy (AUCs=0.81-0.82) across patients. Validation using large-scale electronic health records and in vitro assays further supports the translational relevance of top-ranked candidates. Taking together, STDrug establishes a generalizable framework for incorporating spatial omics into therapeutic discovery, advancing spatially informed and personalized drug repurposing.</t>
+          <t xml:space="preserve">Abstract
+Background:
+Drug discovery remains time-consuming and costly, with most candidates failing before clinical translation. Drug repurposing—identifying new therapeutic indications for approved or investigational compounds—offers a faster and lower-risk alternative by leveraging existing pharmacologic and safety data. Computational approaches, particularly transcriptomics-based strategies that reverse disease-associated gene expression signatures, have shown promise for systematic drug prioritization. However, earlier methods relied primarily on bulk transcriptomic data and overlooked cellular heterogeneity. Recent frameworks incorporating single-cell RNA-seq improved resolution but lack spatial context, which is critical for capturing tissue organization and microenvironmental interactions that influence therapeutic response.
+Objective:
+To address these limitations, we developed STDrug, a computational framework that leverages spatial transcriptomics to enable patient-specific drug repurposing. STDrug identifies disease–normal paired spatial domains and prioritizes candidate therapeutics using pharmacogenomic perturbation data combined with machine learning and large language model–guided gene weighting to estimate drug efficacy, toxicity, and side-effect profiles.
+Methods:
+STDrug consists of three major components: (1) spatial transcriptomic data preprocessing and integration, (2) spatial domain identification, and (3) drug prioritization. Paired diseased and matched normal spatial transcriptomic datasets were harmonized using batch correction and alignment. Spatially informed embeddings were generated using a graph convolutional network built on Harmony-corrected features and spatial coordinates, followed by disease–control balanced clustering to identify paired spatial domains across tissue states. Candidate drugs were prioritized based on their ability to reverse disease-associated gene expression using large-scale perturbation resources (e.g., L1000 and Tahoe-100M). Gene-level importance weights were inferred using a machine learning framework informed by GPT-4o–derived knowledge. Drug scoring further incorporated spatial domain interactions, toxicity profiles from SIDER, and efficacy evidence from the GDSC database to generate patient-specific composite drug scores.
+Results:
+STDrug generated robust patient-level drug prioritization by integrating spatial domain architecture with predicted efficacy and toxicity signals. Across hepatocellular carcinoma and prostate cancer datasets, STDrug outperformed existing single-cell and spatial transcriptomics–based repurposing approaches, achieving improved predictive accuracy (AUC 0.81–0.82). Independent validation using large-scale electronic health record analyses and in vitro experiments supported the translational relevance of top-ranked candidate therapies.
+Conclusions:
+STDrug provides a spatially informed computational framework for precision drug repurposing by integrating spatial transcriptomic structure, transcriptional reversibility, pharmacologic constraints, and machine learning– and generative AI–guided marker prioritization. This approach enables patient-specific therapeutic prediction and offers a scalable strategy for translating spatial transcriptomics into clinical decision support for precision medicine.
+</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -930,13 +941,16 @@
       <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Background
-Postpartum essential hypertension, type 2 diabetes mellitus, and renal disease represent major long-term cardiovascular, metabolic, and renal sequelae of pregnancy that are epidemiologically linked to gestational complications. The objective of this study was to develop a single multi-modality model to simultaneously predict the time to first postpartum onset of these three conditions using routinely collected EHR data.
+Postpartum essential hypertension, type 2 diabetes mellitus, and renal disease represent major long-term cardiovascular, metabolic, and renal sequelae of pregnancy that are epidemiologically linked to gestational complications.
+Objective
+The objective of this study was to develop a single multi-modality model to simultaneously predict the time to first postpartum onset of these three conditions using routinely collected EHR data.
 Methods
-Using Michigan Medicine EHR data (2006–2025) and IRB oversight, we analyzed a cohort of patients with single deliveries and &amp;gt;3 months of postpartum follow-up. The study period began three months postpartum to avoid transient conditions. Our multimodal deep learning framework integrates lab tests, diagnosis codes, and medication codes with demographics. A GRU-D encoder processed temporal numeric data to manage missingness via decay mechanisms. Discrete sequential data were transformed into 1,536-dimensional vectors using LLM model and analyzed with transformer encoders using sinusoidal positional encoding. Predictions from three independent heads were trained via multi-task Cox partial likelihood loss. Performance was evaluated using Harrell’s C-index for discrimination, Integrated Brier Score for calibration, and integrated gradient for modality interpretation.
+Using Michigan Medicine EHR data (2006–2025), we analyzed a cohort of patients with single deliveries and &amp;gt;3 months of postpartum follow-up. The study period began three months postpartum to avoid transient conditions. Our multimodal deep learning framework integrates lab tests, diagnosis codes, and medication codes with demographics. A GRU-D encoder processed temporal numeric data to manage missingness via decay mechanisms. Discrete sequential data were transformed into 1,536-dimensional vectors using LLM model and analyzed with transformer encoders using sinusoidal positional encoding. Predictions from three independent heads were trained via multi-task Cox partial likelihood loss. Performance was evaluated using Harrell’s C-index for discrimination, Integrated Brier Score for calibration, and integrated gradient for modality interpretation.
 Results
-The final analytic cohort was 38486 patients, with delivery years spanning 2006–2025 and a median follow-up of [median] years. The proposed multimodal model achieved mean C-indices of 0.80 ± 0.003 for hypertension, 0.85±0.003 for type 2 diabetes, and 0.79±0.003 for renal disease. Patients in different predicted risk groups show significant disease onset timing. The model consistently outperformed or matched benchmark methods (CoxPH-Lasso, DeepSurv, Random Survival Forest). Modality ablation and permutation importance analysis revealed a clear hierarchy: prenatal diagnosis code carried the dominant predictive signal, followed by lab tests. Medication codes contributed marginal incremental value.
-Conclusion
-A multimodal deep learning framework can accurately and jointly predict the long-term postpartum onset of hypertension, type 2 diabetes, and renal disease. The finding that a labs-plus-diagnoses model captures nearly all discriminative performance, while reducing input complexity, has practical implications for a focused, efficient model deployment.</t>
+The final analytic cohort was 38,486 patients, with delivery years spanning 2006–2025 and a median follow-up of [median] years. The proposed multimodal model achieved mean C-indices of 0.80 ± 0.003 for hypertension, 0.85 ± 0.003 for type 2 diabetes, and 0.79 ± 0.003 for renal disease. Patients in different predicted risk groups show significant disease onset timing. The model consistently outperformed or matched benchmark methods (CoxPH-Lasso, DeepSurv, Random Survival Forest). Modality ablation and permutation importance analysis revealed a clear hierarchy: prenatal diagnosis code carried the dominant predictive signal, followed by lab tests. Medication codes contributed marginal incremental value.
+Conclusions
+A multimodal deep learning framework can accurately and jointly predict the long-term postpartum onset of hypertension, type 2 diabetes, and renal disease. The finding that a labs-plus-diagnoses model captures nearly all discriminative performance, while reducing input complexity, has practical implications for a focused, efficient model deployment.
+"</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -1079,10 +1093,16 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Background: Spatial omics enables the integration of high-dimensional molecular organization with clinical outcomes. However, incorporating spatial single-cell information into predictive models at the population scale remains a significant challenge.
-Methods: To address this, we adapted BSNMani (Bayesian Scalar-on-Network regression with Manifold learning). This framework is designed to integrate subject-specific, spatially informed gene co-expression networks directly into clinical prediction models. We evaluated the framework's predictive performance and ability to utilize cell-type-specific spatial omics data to enhance analytical granularity.
-Results: In benchmark comparisons, feature selection using BSNMani significantly outperformed both Elastic Net and Lasso methods. When applied to the SEA-AD MERFISH transcriptomics cohort, the framework achieved an accuracy of 0.74 for Alzheimer’s disease (AD) prediction. It successfully revealed four distinct gene–gene co-expression subnetworks with clear biological relevance, including pathways related to glutamatergic synapses and neurogenesis. Furthermore, BSNMani achieved strong survival prediction in a separate breast cancer cohort measured by Imaging Mass Cytometry (IMC) (C-index = 0.77), identifying two key prognostic subnetworks.
-Conclusions: BSNMani is a powerful, highly interpretable tool that leverages high-dimensional, cell-type-specific spatial omics data for clinical outcome prediction. It scales effectively to population-level analyses across diverse disease settings, revealing deep biological insights while maintaining easy interpretation for clinical application.</t>
+          <t>Background
+Spatial omics enables the integration of high-dimensional molecular organization with clinical outcomes, yet incorporating spatial single-cell information into predictive models at the population scale remains a significant challenge. Current analytical methods predominantly focus on single-sample analyses, limiting the translational potential of spatial omics for treatment stratification, prognosis, and disease risk prediction.
+Objective
+To adapt and evaluate BSNMani (Bayesian Scalar-on-Network regression with Manifold learning) for integrating subject-specific, spatially informed gene co-expression networks into clinical prediction models, and to demonstrate its utility and interpretability across diverse single-cell spatial omics modalities and disease cohorts.
+Methods
+Subject-specific, spatially aware gene co-expression matrices were constructed from single-cell spatial transcriptomics and proteomics data. The BSNMani framework was applied to decompose these high-dimensional networks into low-rank representations on a Stiefel manifold, utilizing the resulting subnetwork loadings as predictors in clinical regression and survival models. The predictive performance of BSNMani was evaluated using leave-one-out cross-validation with nonparametric bootstrapping and benchmarked against classical high-dimensional feature extraction methods, including Elastic Net and Lasso.
+Results
+In benchmark comparisons, BSNMani significantly outperformed both Elastic Net and Lasso in predictive performance. When applied to the SEA-AD MERFISH transcriptomics cohort, the BSNMani framework achieved an AUC of 0.76 for Alzheimer’s disease prediction. It successfully revealed four distinct gene–gene co-expression subnetworks with clear biological relevance, capturing pathways related to glutamatergic synapses and neurogenesis. In a separate breast cancer cohort measured by Imaging Mass Cytometry (IMC), BSNMani achieved strong survival prediction (C-index = 0.776), identifying two key prognostic subnetworks driven by distinct hub markers, including EGFR and ERBB2. Furthermore, application to cell-type-specific spatial data demonstrated the framework's ability to enhance analytical granularity and pinpoint localized biological patterns.
+Conclusions
+BSNMani is a powerful, highly interpretable tool that leverages high-dimensional, cell-type-specific spatial omics data for clinical outcome prediction. By mathematically capturing complex network topologies, it scales effectively to population-level analyses across diverse disease settings, revealing deep biological insights while maintaining transparency for clinical application.</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -1929,7 +1949,42 @@
       </c>
     </row>
     <row r="31">
-      <c r="G31" s="8" t="n"/>
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>SCG: Spatially Co-Expressed Gene Identification through Spatially Varying Networks</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Ihsan E. Buker, Yang Ni, Jian Kang, Stephanie Hicks, Satwik Acharyya</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Department of Biostatistics, School of Public Health, University of Alabama at Birmingham, Birmingham, AL, USA;
+Department of Statistics and Data Sciences, College of Natural Sciences, The University of Texas at Austin, Austin, TX, USA;
+Department of Biostatistics, School of Public Health, University of Michigan, Ann Arbor, MI, USA;
+Department of Biostatistics, Bloomberg School of Public Health, Johns Hopkins University, Baltimore, MD, USA;</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>iebuker@uab.edu</t>
+        </is>
+      </c>
+      <c r="G31" s="8" t="inlineStr">
+        <is>
+          <t>Background: Spatial transcriptomics (ST) profiling technologies provide high-resolution maps of gene expression across tissues, revealing the spatial organization of cells and the tissue microenvironment. These advances necessitate statistical frameworks for characterizing spatially heterogeneous gene association networks that contribute to disease etiology. We introduce the novel concept of Spatially Coexpressed Genes (SCGs), which provides a high-resolution spatial map of gene-gene co-expression and enables the study of spot-specific gene networks, offering new insights into spatially resolved mechanisms of disease.
+Methods: To identify SCGs, we propose a spatial covariance regression (SCR) model that learns spatially varying marginal dependence from high-resolution ST data while exploiting low-rank structure. SCR models location-specific covariance matrices using a spatially varying factor model whose loadings are decomposed into a global loadings matrix and a set of spatial basis functions. We impose a multiplicative gamma process shrinkage prior on the global loadings to encourage sparsity and low-rank structure and assign Gaussian process priors with rational quadratic kernels to the spatial basis functions to capture latent spatial variation. SCGs are identified via Otsu‚Äôs thresholding applied to the spatial variation of estimated edges. To ensure scalable inference, we develop a GPU-accelerated variational Bayes algorithm. We assess the performance of SCR through extensive simulation studies and demonstrate its application to two datasets: Visium-based breast cancer data and Xenium-based Alzheimer‚Äôs mouse-brain data.
+Results: We simulated spatial fields of 10,000‚Äì50,000 locations for 30 genes and summarized results over 20 replicates. We observed high values of Matthews correlation coefficients (MCC: 0.94‚Äì0.95) and true positive rates (TPR: 0.94‚Äì0.97), accompanied by consistently low false positive rates (FPR &lt; 0.01). These results indicate effective classification between true and spurious edges despite class imbalance induced in the data simulation. We evaluated the performance of SCR in estimating spatially varying edges using the RV coefficient. An RV value close to 1 (or 0) indicates concordance (or discordance) between the estimated and true spatial edges. On average, the RV coefficients were close to 1 across all spatial locations and replicates. Regarding scalability, our method requires approximately 5 hours to estimate spatially resolved networks across 50,000 locations.
+Conclusions: We developed a GPU-accelerated CAVI algorithm that enables scalable inference of spatial gene networks at tens of thousands of locations. Overall, the SCR framework provides a practical and statistically principled approach for characterizing spatially varying gene co-expression, opening new avenues for studying spatial mechanisms in disease etiology.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="G32" s="8" t="n"/>
@@ -1953,7 +2008,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC30"/>
+  <dimension ref="A1:AC31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3721,6 +3776,41 @@
       <c r="AB30" s="14" t="n"/>
       <c r="AC30" s="14" t="n"/>
     </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>31</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>SCG: Spatially Co-Expressed Gene Identification through Spatially Varying Networks</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Garmire, Lana</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Osborne, John D</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>Chen, Jake Y</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:AC30"/>
   <dataValidations count="1">

</xml_diff>

<commit_message>
Add Chong Zechen as 4th reviewer; backup workbook; restore Blazer PIN
- Backup saved as *_BACKUP_before_adding_Zechen.xlsx (3 reviewers only)
- Main workbook: Reviewer 4 column set to Chong, Zechen for all abstracts; cols 5/10/15 unchanged (Lana slots preserved)
- shared_review_portal: add DEFAULT password for Chong, Zechen
- Script add_zechen_reviewer.py documents the change

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/ATTIS abstract submission_April 21, 2026_09.24_with_review_assignments.xlsx
+++ b/ATTIS abstract submission_April 21, 2026_09.24_with_review_assignments.xlsx
@@ -2233,7 +2233,11 @@
       <c r="Q2" s="14" t="n"/>
       <c r="R2" s="14" t="n"/>
       <c r="S2" s="14" t="n"/>
-      <c r="T2" s="14" t="n"/>
+      <c r="T2" s="14" t="inlineStr">
+        <is>
+          <t>Chong, Zechen</t>
+        </is>
+      </c>
       <c r="U2" s="14" t="n"/>
       <c r="V2" s="14" t="n"/>
       <c r="W2" s="14" t="n"/>
@@ -2288,7 +2292,11 @@
       <c r="Q3" s="14" t="n"/>
       <c r="R3" s="14" t="n"/>
       <c r="S3" s="14" t="n"/>
-      <c r="T3" s="14" t="n"/>
+      <c r="T3" s="14" t="inlineStr">
+        <is>
+          <t>Chong, Zechen</t>
+        </is>
+      </c>
       <c r="U3" s="14" t="n"/>
       <c r="V3" s="14" t="n"/>
       <c r="W3" s="14" t="n"/>
@@ -2339,7 +2347,11 @@
       <c r="Q4" s="14" t="n"/>
       <c r="R4" s="14" t="n"/>
       <c r="S4" s="14" t="n"/>
-      <c r="T4" s="14" t="n"/>
+      <c r="T4" s="14" t="inlineStr">
+        <is>
+          <t>Chong, Zechen</t>
+        </is>
+      </c>
       <c r="U4" s="14" t="n"/>
       <c r="V4" s="14" t="n"/>
       <c r="W4" s="14" t="n"/>
@@ -2394,7 +2406,11 @@
       <c r="Q5" s="14" t="n"/>
       <c r="R5" s="14" t="n"/>
       <c r="S5" s="14" t="n"/>
-      <c r="T5" s="14" t="n"/>
+      <c r="T5" s="14" t="inlineStr">
+        <is>
+          <t>Chong, Zechen</t>
+        </is>
+      </c>
       <c r="U5" s="14" t="n"/>
       <c r="V5" s="14" t="n"/>
       <c r="W5" s="14" t="n"/>
@@ -2449,7 +2465,11 @@
       <c r="Q6" s="14" t="n"/>
       <c r="R6" s="14" t="n"/>
       <c r="S6" s="14" t="n"/>
-      <c r="T6" s="14" t="n"/>
+      <c r="T6" s="14" t="inlineStr">
+        <is>
+          <t>Chong, Zechen</t>
+        </is>
+      </c>
       <c r="U6" s="14" t="n"/>
       <c r="V6" s="14" t="n"/>
       <c r="W6" s="14" t="n"/>
@@ -2504,7 +2524,11 @@
       <c r="Q7" s="14" t="n"/>
       <c r="R7" s="14" t="n"/>
       <c r="S7" s="14" t="n"/>
-      <c r="T7" s="14" t="n"/>
+      <c r="T7" s="14" t="inlineStr">
+        <is>
+          <t>Chong, Zechen</t>
+        </is>
+      </c>
       <c r="U7" s="14" t="n"/>
       <c r="V7" s="14" t="n"/>
       <c r="W7" s="14" t="n"/>
@@ -2559,7 +2583,11 @@
       <c r="Q8" s="14" t="n"/>
       <c r="R8" s="14" t="n"/>
       <c r="S8" s="14" t="n"/>
-      <c r="T8" s="14" t="n"/>
+      <c r="T8" s="14" t="inlineStr">
+        <is>
+          <t>Chong, Zechen</t>
+        </is>
+      </c>
       <c r="U8" s="14" t="n"/>
       <c r="V8" s="14" t="n"/>
       <c r="W8" s="14" t="n"/>
@@ -2614,7 +2642,11 @@
       <c r="Q9" s="14" t="n"/>
       <c r="R9" s="14" t="n"/>
       <c r="S9" s="14" t="n"/>
-      <c r="T9" s="14" t="n"/>
+      <c r="T9" s="14" t="inlineStr">
+        <is>
+          <t>Chong, Zechen</t>
+        </is>
+      </c>
       <c r="U9" s="14" t="n"/>
       <c r="V9" s="14" t="n"/>
       <c r="W9" s="14" t="n"/>
@@ -2669,7 +2701,11 @@
       <c r="Q10" s="14" t="n"/>
       <c r="R10" s="14" t="n"/>
       <c r="S10" s="14" t="n"/>
-      <c r="T10" s="14" t="n"/>
+      <c r="T10" s="14" t="inlineStr">
+        <is>
+          <t>Chong, Zechen</t>
+        </is>
+      </c>
       <c r="U10" s="14" t="n"/>
       <c r="V10" s="14" t="n"/>
       <c r="W10" s="14" t="n"/>
@@ -2724,7 +2760,11 @@
       <c r="Q11" s="14" t="n"/>
       <c r="R11" s="14" t="n"/>
       <c r="S11" s="14" t="n"/>
-      <c r="T11" s="14" t="n"/>
+      <c r="T11" s="14" t="inlineStr">
+        <is>
+          <t>Chong, Zechen</t>
+        </is>
+      </c>
       <c r="U11" s="14" t="n"/>
       <c r="V11" s="14" t="n"/>
       <c r="W11" s="14" t="n"/>
@@ -2775,7 +2815,11 @@
       <c r="Q12" s="14" t="n"/>
       <c r="R12" s="14" t="n"/>
       <c r="S12" s="14" t="n"/>
-      <c r="T12" s="14" t="n"/>
+      <c r="T12" s="14" t="inlineStr">
+        <is>
+          <t>Chong, Zechen</t>
+        </is>
+      </c>
       <c r="U12" s="14" t="n"/>
       <c r="V12" s="14" t="n"/>
       <c r="W12" s="14" t="n"/>
@@ -2830,7 +2874,11 @@
       <c r="Q13" s="14" t="n"/>
       <c r="R13" s="14" t="n"/>
       <c r="S13" s="14" t="n"/>
-      <c r="T13" s="14" t="n"/>
+      <c r="T13" s="14" t="inlineStr">
+        <is>
+          <t>Chong, Zechen</t>
+        </is>
+      </c>
       <c r="U13" s="14" t="n"/>
       <c r="V13" s="14" t="n"/>
       <c r="W13" s="14" t="n"/>
@@ -2885,7 +2933,11 @@
       <c r="Q14" s="14" t="n"/>
       <c r="R14" s="14" t="n"/>
       <c r="S14" s="14" t="n"/>
-      <c r="T14" s="14" t="n"/>
+      <c r="T14" s="14" t="inlineStr">
+        <is>
+          <t>Chong, Zechen</t>
+        </is>
+      </c>
       <c r="U14" s="14" t="n"/>
       <c r="V14" s="14" t="n"/>
       <c r="W14" s="14" t="n"/>
@@ -2940,7 +2992,11 @@
       <c r="Q15" s="14" t="n"/>
       <c r="R15" s="14" t="n"/>
       <c r="S15" s="14" t="n"/>
-      <c r="T15" s="14" t="n"/>
+      <c r="T15" s="14" t="inlineStr">
+        <is>
+          <t>Chong, Zechen</t>
+        </is>
+      </c>
       <c r="U15" s="14" t="n"/>
       <c r="V15" s="14" t="n"/>
       <c r="W15" s="14" t="n"/>
@@ -2995,7 +3051,11 @@
       <c r="Q16" s="14" t="n"/>
       <c r="R16" s="14" t="n"/>
       <c r="S16" s="14" t="n"/>
-      <c r="T16" s="14" t="n"/>
+      <c r="T16" s="14" t="inlineStr">
+        <is>
+          <t>Chong, Zechen</t>
+        </is>
+      </c>
       <c r="U16" s="14" t="n"/>
       <c r="V16" s="14" t="n"/>
       <c r="W16" s="14" t="n"/>
@@ -3050,7 +3110,11 @@
       <c r="Q17" s="14" t="n"/>
       <c r="R17" s="14" t="n"/>
       <c r="S17" s="14" t="n"/>
-      <c r="T17" s="14" t="n"/>
+      <c r="T17" s="14" t="inlineStr">
+        <is>
+          <t>Chong, Zechen</t>
+        </is>
+      </c>
       <c r="U17" s="14" t="n"/>
       <c r="V17" s="14" t="n"/>
       <c r="W17" s="14" t="n"/>
@@ -3105,7 +3169,11 @@
       <c r="Q18" s="14" t="n"/>
       <c r="R18" s="14" t="n"/>
       <c r="S18" s="14" t="n"/>
-      <c r="T18" s="14" t="n"/>
+      <c r="T18" s="14" t="inlineStr">
+        <is>
+          <t>Chong, Zechen</t>
+        </is>
+      </c>
       <c r="U18" s="14" t="n"/>
       <c r="V18" s="14" t="n"/>
       <c r="W18" s="14" t="n"/>
@@ -3160,7 +3228,11 @@
       <c r="Q19" s="14" t="n"/>
       <c r="R19" s="14" t="n"/>
       <c r="S19" s="14" t="n"/>
-      <c r="T19" s="14" t="n"/>
+      <c r="T19" s="14" t="inlineStr">
+        <is>
+          <t>Chong, Zechen</t>
+        </is>
+      </c>
       <c r="U19" s="14" t="n"/>
       <c r="V19" s="14" t="n"/>
       <c r="W19" s="14" t="n"/>
@@ -3215,7 +3287,11 @@
       <c r="Q20" s="14" t="n"/>
       <c r="R20" s="14" t="n"/>
       <c r="S20" s="14" t="n"/>
-      <c r="T20" s="14" t="n"/>
+      <c r="T20" s="14" t="inlineStr">
+        <is>
+          <t>Chong, Zechen</t>
+        </is>
+      </c>
       <c r="U20" s="14" t="n"/>
       <c r="V20" s="14" t="n"/>
       <c r="W20" s="14" t="n"/>
@@ -3270,7 +3346,11 @@
       <c r="Q21" s="14" t="n"/>
       <c r="R21" s="14" t="n"/>
       <c r="S21" s="14" t="n"/>
-      <c r="T21" s="14" t="n"/>
+      <c r="T21" s="14" t="inlineStr">
+        <is>
+          <t>Chong, Zechen</t>
+        </is>
+      </c>
       <c r="U21" s="14" t="n"/>
       <c r="V21" s="14" t="n"/>
       <c r="W21" s="14" t="n"/>
@@ -3325,7 +3405,11 @@
       <c r="Q22" s="14" t="n"/>
       <c r="R22" s="14" t="n"/>
       <c r="S22" s="14" t="n"/>
-      <c r="T22" s="14" t="n"/>
+      <c r="T22" s="14" t="inlineStr">
+        <is>
+          <t>Chong, Zechen</t>
+        </is>
+      </c>
       <c r="U22" s="14" t="n"/>
       <c r="V22" s="14" t="n"/>
       <c r="W22" s="14" t="n"/>
@@ -3380,7 +3464,11 @@
       <c r="Q23" s="14" t="n"/>
       <c r="R23" s="14" t="n"/>
       <c r="S23" s="14" t="n"/>
-      <c r="T23" s="14" t="n"/>
+      <c r="T23" s="14" t="inlineStr">
+        <is>
+          <t>Chong, Zechen</t>
+        </is>
+      </c>
       <c r="U23" s="14" t="n"/>
       <c r="V23" s="14" t="n"/>
       <c r="W23" s="14" t="n"/>
@@ -3435,7 +3523,11 @@
       <c r="Q24" s="14" t="n"/>
       <c r="R24" s="14" t="n"/>
       <c r="S24" s="14" t="n"/>
-      <c r="T24" s="14" t="n"/>
+      <c r="T24" s="14" t="inlineStr">
+        <is>
+          <t>Chong, Zechen</t>
+        </is>
+      </c>
       <c r="U24" s="14" t="n"/>
       <c r="V24" s="14" t="n"/>
       <c r="W24" s="14" t="n"/>
@@ -3490,7 +3582,11 @@
       <c r="Q25" s="14" t="n"/>
       <c r="R25" s="14" t="n"/>
       <c r="S25" s="14" t="n"/>
-      <c r="T25" s="14" t="n"/>
+      <c r="T25" s="14" t="inlineStr">
+        <is>
+          <t>Chong, Zechen</t>
+        </is>
+      </c>
       <c r="U25" s="14" t="n"/>
       <c r="V25" s="14" t="n"/>
       <c r="W25" s="14" t="n"/>
@@ -3545,7 +3641,11 @@
       <c r="Q26" s="14" t="n"/>
       <c r="R26" s="14" t="n"/>
       <c r="S26" s="14" t="n"/>
-      <c r="T26" s="14" t="n"/>
+      <c r="T26" s="14" t="inlineStr">
+        <is>
+          <t>Chong, Zechen</t>
+        </is>
+      </c>
       <c r="U26" s="14" t="n"/>
       <c r="V26" s="14" t="n"/>
       <c r="W26" s="14" t="n"/>
@@ -3600,7 +3700,11 @@
       <c r="Q27" s="14" t="n"/>
       <c r="R27" s="14" t="n"/>
       <c r="S27" s="14" t="n"/>
-      <c r="T27" s="14" t="n"/>
+      <c r="T27" s="14" t="inlineStr">
+        <is>
+          <t>Chong, Zechen</t>
+        </is>
+      </c>
       <c r="U27" s="14" t="n"/>
       <c r="V27" s="14" t="n"/>
       <c r="W27" s="14" t="n"/>
@@ -3655,7 +3759,11 @@
       <c r="Q28" s="14" t="n"/>
       <c r="R28" s="14" t="n"/>
       <c r="S28" s="14" t="n"/>
-      <c r="T28" s="14" t="n"/>
+      <c r="T28" s="14" t="inlineStr">
+        <is>
+          <t>Chong, Zechen</t>
+        </is>
+      </c>
       <c r="U28" s="14" t="n"/>
       <c r="V28" s="14" t="n"/>
       <c r="W28" s="14" t="n"/>
@@ -3710,7 +3818,11 @@
       <c r="Q29" s="14" t="n"/>
       <c r="R29" s="14" t="n"/>
       <c r="S29" s="14" t="n"/>
-      <c r="T29" s="14" t="n"/>
+      <c r="T29" s="14" t="inlineStr">
+        <is>
+          <t>Chong, Zechen</t>
+        </is>
+      </c>
       <c r="U29" s="14" t="n"/>
       <c r="V29" s="14" t="n"/>
       <c r="W29" s="14" t="n"/>
@@ -3765,7 +3877,11 @@
       <c r="Q30" s="14" t="n"/>
       <c r="R30" s="14" t="n"/>
       <c r="S30" s="14" t="n"/>
-      <c r="T30" s="14" t="n"/>
+      <c r="T30" s="14" t="inlineStr">
+        <is>
+          <t>Chong, Zechen</t>
+        </is>
+      </c>
       <c r="U30" s="14" t="n"/>
       <c r="V30" s="14" t="n"/>
       <c r="W30" s="14" t="n"/>
@@ -3808,6 +3924,11 @@
       <c r="O31" t="inlineStr">
         <is>
           <t>Chen, Jake Y</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>Chong, Zechen</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Randomize non-Lana reviewer slots; backup before randomize; preserve Lana placements
- Cells with Garmire, Lana unchanged (same 13 abstract slots)
- Other reviewer columns (5,10,15,20) re-sampled without duplication; Lana not placed in flex slots

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/ATTIS abstract submission_April 21, 2026_09.24_with_review_assignments.xlsx
+++ b/ATTIS abstract submission_April 21, 2026_09.24_with_review_assignments.xlsx
@@ -2208,7 +2208,7 @@
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>Amy Wang</t>
+          <t>Osborne, John D</t>
         </is>
       </c>
       <c r="F2" s="14" t="n"/>
@@ -2217,7 +2217,7 @@
       <c r="I2" s="14" t="n"/>
       <c r="J2" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="K2" s="14" t="n"/>
@@ -2235,7 +2235,7 @@
       <c r="S2" s="14" t="n"/>
       <c r="T2" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="U2" s="14" t="n"/>
@@ -2267,7 +2267,7 @@
       </c>
       <c r="E3" s="14" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Osborne, John D</t>
         </is>
       </c>
       <c r="F3" s="14" t="n"/>
@@ -2276,7 +2276,7 @@
       <c r="I3" s="14" t="n"/>
       <c r="J3" s="14" t="inlineStr">
         <is>
-          <t>Mosa, Abu S</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="K3" s="14" t="n"/>
@@ -2285,7 +2285,7 @@
       <c r="N3" s="14" t="n"/>
       <c r="O3" s="14" t="inlineStr">
         <is>
-          <t>Osborne, John D</t>
+          <t>Chong, Zechen</t>
         </is>
       </c>
       <c r="P3" s="14" t="n"/>
@@ -2294,7 +2294,7 @@
       <c r="S3" s="14" t="n"/>
       <c r="T3" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="U3" s="14" t="n"/>
@@ -2322,7 +2322,7 @@
       </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="F4" s="14" t="n"/>
@@ -2331,7 +2331,7 @@
       <c r="I4" s="14" t="n"/>
       <c r="J4" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jin (Campus)</t>
+          <t>Chong, Zechen</t>
         </is>
       </c>
       <c r="K4" s="14" t="n"/>
@@ -2349,7 +2349,7 @@
       <c r="S4" s="14" t="n"/>
       <c r="T4" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="U4" s="14" t="n"/>
@@ -2381,7 +2381,7 @@
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="F5" s="14" t="n"/>
@@ -2390,7 +2390,7 @@
       <c r="I5" s="14" t="n"/>
       <c r="J5" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jin (Campus)</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="K5" s="14" t="n"/>
@@ -2399,7 +2399,7 @@
       <c r="N5" s="14" t="n"/>
       <c r="O5" s="14" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Chong, Zechen</t>
         </is>
       </c>
       <c r="P5" s="14" t="n"/>
@@ -2408,7 +2408,7 @@
       <c r="S5" s="14" t="n"/>
       <c r="T5" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="U5" s="14" t="n"/>
@@ -2440,7 +2440,7 @@
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
-          <t>Mosa, Abu S</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="F6" s="14" t="n"/>
@@ -2449,7 +2449,7 @@
       <c r="I6" s="14" t="n"/>
       <c r="J6" s="14" t="inlineStr">
         <is>
-          <t>Osborne, John D</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="K6" s="14" t="n"/>
@@ -2458,7 +2458,7 @@
       <c r="N6" s="14" t="n"/>
       <c r="O6" s="14" t="inlineStr">
         <is>
-          <t>Amy Wang</t>
+          <t>Chong, Zechen</t>
         </is>
       </c>
       <c r="P6" s="14" t="n"/>
@@ -2467,7 +2467,7 @@
       <c r="S6" s="14" t="n"/>
       <c r="T6" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="U6" s="14" t="n"/>
@@ -2499,7 +2499,7 @@
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Chong, Zechen</t>
         </is>
       </c>
       <c r="F7" s="14" t="n"/>
@@ -2508,7 +2508,7 @@
       <c r="I7" s="14" t="n"/>
       <c r="J7" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jin (Campus)</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="K7" s="14" t="n"/>
@@ -2517,7 +2517,7 @@
       <c r="N7" s="14" t="n"/>
       <c r="O7" s="14" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Osborne, John D</t>
         </is>
       </c>
       <c r="P7" s="14" t="n"/>
@@ -2526,7 +2526,7 @@
       <c r="S7" s="14" t="n"/>
       <c r="T7" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="U7" s="14" t="n"/>
@@ -2558,7 +2558,7 @@
       </c>
       <c r="E8" s="14" t="inlineStr">
         <is>
-          <t>Mosa, Abu S</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="F8" s="14" t="n"/>
@@ -2567,7 +2567,7 @@
       <c r="I8" s="14" t="n"/>
       <c r="J8" s="14" t="inlineStr">
         <is>
-          <t>Osborne, John D</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="K8" s="14" t="n"/>
@@ -2576,7 +2576,7 @@
       <c r="N8" s="14" t="n"/>
       <c r="O8" s="14" t="inlineStr">
         <is>
-          <t>Amy Wang</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="P8" s="14" t="n"/>
@@ -2617,7 +2617,7 @@
       </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
-          <t>Mosa, Abu S</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="F9" s="14" t="n"/>
@@ -2626,7 +2626,7 @@
       <c r="I9" s="14" t="n"/>
       <c r="J9" s="14" t="inlineStr">
         <is>
-          <t>Osborne, John D</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="K9" s="14" t="n"/>
@@ -2635,7 +2635,7 @@
       <c r="N9" s="14" t="n"/>
       <c r="O9" s="14" t="inlineStr">
         <is>
-          <t>Amy Wang</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="P9" s="14" t="n"/>
@@ -2644,7 +2644,7 @@
       <c r="S9" s="14" t="n"/>
       <c r="T9" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="U9" s="14" t="n"/>
@@ -2676,7 +2676,7 @@
       </c>
       <c r="E10" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="F10" s="14" t="n"/>
@@ -2685,7 +2685,7 @@
       <c r="I10" s="14" t="n"/>
       <c r="J10" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jin (Campus)</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="K10" s="14" t="n"/>
@@ -2694,7 +2694,7 @@
       <c r="N10" s="14" t="n"/>
       <c r="O10" s="14" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="P10" s="14" t="n"/>
@@ -2703,7 +2703,7 @@
       <c r="S10" s="14" t="n"/>
       <c r="T10" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="U10" s="14" t="n"/>
@@ -2735,7 +2735,7 @@
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
-          <t>Mosa, Abu S</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="F11" s="14" t="n"/>
@@ -2744,7 +2744,7 @@
       <c r="I11" s="14" t="n"/>
       <c r="J11" s="14" t="inlineStr">
         <is>
-          <t>Osborne, John D</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="K11" s="14" t="n"/>
@@ -2753,7 +2753,7 @@
       <c r="N11" s="14" t="n"/>
       <c r="O11" s="14" t="inlineStr">
         <is>
-          <t>Amy Wang</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="P11" s="14" t="n"/>
@@ -2762,7 +2762,7 @@
       <c r="S11" s="14" t="n"/>
       <c r="T11" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="U11" s="14" t="n"/>
@@ -2790,7 +2790,7 @@
       </c>
       <c r="E12" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jin (Campus)</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="F12" s="14" t="n"/>
@@ -2817,7 +2817,7 @@
       <c r="S12" s="14" t="n"/>
       <c r="T12" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="U12" s="14" t="n"/>
@@ -2849,7 +2849,7 @@
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>Osborne, John D</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="F13" s="14" t="n"/>
@@ -2858,7 +2858,7 @@
       <c r="I13" s="14" t="n"/>
       <c r="J13" s="14" t="inlineStr">
         <is>
-          <t>Amy Wang</t>
+          <t>Osborne, John D</t>
         </is>
       </c>
       <c r="K13" s="14" t="n"/>
@@ -2867,7 +2867,7 @@
       <c r="N13" s="14" t="n"/>
       <c r="O13" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="P13" s="14" t="n"/>
@@ -2876,7 +2876,7 @@
       <c r="S13" s="14" t="n"/>
       <c r="T13" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="U13" s="14" t="n"/>
@@ -2917,7 +2917,7 @@
       <c r="I14" s="14" t="n"/>
       <c r="J14" s="14" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Chong, Zechen</t>
         </is>
       </c>
       <c r="K14" s="14" t="n"/>
@@ -2926,7 +2926,7 @@
       <c r="N14" s="14" t="n"/>
       <c r="O14" s="14" t="inlineStr">
         <is>
-          <t>Mosa, Abu S</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="P14" s="14" t="n"/>
@@ -2935,7 +2935,7 @@
       <c r="S14" s="14" t="n"/>
       <c r="T14" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="U14" s="14" t="n"/>
@@ -2967,7 +2967,7 @@
       </c>
       <c r="E15" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jin (Campus)</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="F15" s="14" t="n"/>
@@ -2985,7 +2985,7 @@
       <c r="N15" s="14" t="n"/>
       <c r="O15" s="14" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="P15" s="14" t="n"/>
@@ -3035,7 +3035,7 @@
       <c r="I16" s="14" t="n"/>
       <c r="J16" s="14" t="inlineStr">
         <is>
-          <t>Amy Wang</t>
+          <t>Chong, Zechen</t>
         </is>
       </c>
       <c r="K16" s="14" t="n"/>
@@ -3044,7 +3044,7 @@
       <c r="N16" s="14" t="n"/>
       <c r="O16" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="P16" s="14" t="n"/>
@@ -3053,7 +3053,7 @@
       <c r="S16" s="14" t="n"/>
       <c r="T16" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="U16" s="14" t="n"/>
@@ -3085,7 +3085,7 @@
       </c>
       <c r="E17" s="14" t="inlineStr">
         <is>
-          <t>Amy Wang</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="F17" s="14" t="n"/>
@@ -3094,7 +3094,7 @@
       <c r="I17" s="14" t="n"/>
       <c r="J17" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Osborne, John D</t>
         </is>
       </c>
       <c r="K17" s="14" t="n"/>
@@ -3103,7 +3103,7 @@
       <c r="N17" s="14" t="n"/>
       <c r="O17" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jin (Campus)</t>
+          <t>Chong, Zechen</t>
         </is>
       </c>
       <c r="P17" s="14" t="n"/>
@@ -3112,7 +3112,7 @@
       <c r="S17" s="14" t="n"/>
       <c r="T17" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="U17" s="14" t="n"/>
@@ -3144,7 +3144,7 @@
       </c>
       <c r="E18" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Chong, Zechen</t>
         </is>
       </c>
       <c r="F18" s="14" t="n"/>
@@ -3153,7 +3153,7 @@
       <c r="I18" s="14" t="n"/>
       <c r="J18" s="14" t="inlineStr">
         <is>
-          <t>Mosa, Abu S</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="K18" s="14" t="n"/>
@@ -3162,7 +3162,7 @@
       <c r="N18" s="14" t="n"/>
       <c r="O18" s="14" t="inlineStr">
         <is>
-          <t>Osborne, John D</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="P18" s="14" t="n"/>
@@ -3171,7 +3171,7 @@
       <c r="S18" s="14" t="n"/>
       <c r="T18" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="U18" s="14" t="n"/>
@@ -3203,7 +3203,7 @@
       </c>
       <c r="E19" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Chong, Zechen</t>
         </is>
       </c>
       <c r="F19" s="14" t="n"/>
@@ -3221,7 +3221,7 @@
       <c r="N19" s="14" t="n"/>
       <c r="O19" s="14" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="P19" s="14" t="n"/>
@@ -3230,7 +3230,7 @@
       <c r="S19" s="14" t="n"/>
       <c r="T19" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="U19" s="14" t="n"/>
@@ -3271,7 +3271,7 @@
       <c r="I20" s="14" t="n"/>
       <c r="J20" s="14" t="inlineStr">
         <is>
-          <t>Osborne, John D</t>
+          <t>Chong, Zechen</t>
         </is>
       </c>
       <c r="K20" s="14" t="n"/>
@@ -3289,7 +3289,7 @@
       <c r="S20" s="14" t="n"/>
       <c r="T20" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="U20" s="14" t="n"/>
@@ -3330,7 +3330,7 @@
       <c r="I21" s="14" t="n"/>
       <c r="J21" s="14" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="K21" s="14" t="n"/>
@@ -3339,7 +3339,7 @@
       <c r="N21" s="14" t="n"/>
       <c r="O21" s="14" t="inlineStr">
         <is>
-          <t>Mosa, Abu S</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="P21" s="14" t="n"/>
@@ -3348,7 +3348,7 @@
       <c r="S21" s="14" t="n"/>
       <c r="T21" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Osborne, John D</t>
         </is>
       </c>
       <c r="U21" s="14" t="n"/>
@@ -3380,7 +3380,7 @@
       </c>
       <c r="E22" s="14" t="inlineStr">
         <is>
-          <t>Osborne, John D</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="F22" s="14" t="n"/>
@@ -3389,7 +3389,7 @@
       <c r="I22" s="14" t="n"/>
       <c r="J22" s="14" t="inlineStr">
         <is>
-          <t>Amy Wang</t>
+          <t>Osborne, John D</t>
         </is>
       </c>
       <c r="K22" s="14" t="n"/>
@@ -3398,7 +3398,7 @@
       <c r="N22" s="14" t="n"/>
       <c r="O22" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jin (Campus)</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="P22" s="14" t="n"/>
@@ -3407,7 +3407,7 @@
       <c r="S22" s="14" t="n"/>
       <c r="T22" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="U22" s="14" t="n"/>
@@ -3448,7 +3448,7 @@
       <c r="I23" s="14" t="n"/>
       <c r="J23" s="14" t="inlineStr">
         <is>
-          <t>Mosa, Abu S</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="K23" s="14" t="n"/>
@@ -3457,7 +3457,7 @@
       <c r="N23" s="14" t="n"/>
       <c r="O23" s="14" t="inlineStr">
         <is>
-          <t>Osborne, John D</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="P23" s="14" t="n"/>
@@ -3466,7 +3466,7 @@
       <c r="S23" s="14" t="n"/>
       <c r="T23" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="U23" s="14" t="n"/>
@@ -3516,7 +3516,7 @@
       <c r="N24" s="14" t="n"/>
       <c r="O24" s="14" t="inlineStr">
         <is>
-          <t>Mosa, Abu S</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="P24" s="14" t="n"/>
@@ -3525,7 +3525,7 @@
       <c r="S24" s="14" t="n"/>
       <c r="T24" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="U24" s="14" t="n"/>
@@ -3557,7 +3557,7 @@
       </c>
       <c r="E25" s="14" t="inlineStr">
         <is>
-          <t>Osborne, John D</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="F25" s="14" t="n"/>
@@ -3575,7 +3575,7 @@
       <c r="N25" s="14" t="n"/>
       <c r="O25" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jin (Campus)</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="P25" s="14" t="n"/>
@@ -3584,7 +3584,7 @@
       <c r="S25" s="14" t="n"/>
       <c r="T25" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="U25" s="14" t="n"/>
@@ -3625,7 +3625,7 @@
       <c r="I26" s="14" t="n"/>
       <c r="J26" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jin (Campus)</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="K26" s="14" t="n"/>
@@ -3643,7 +3643,7 @@
       <c r="S26" s="14" t="n"/>
       <c r="T26" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="U26" s="14" t="n"/>
@@ -3693,7 +3693,7 @@
       <c r="N27" s="14" t="n"/>
       <c r="O27" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="P27" s="14" t="n"/>
@@ -3743,7 +3743,7 @@
       <c r="I28" s="14" t="n"/>
       <c r="J28" s="14" t="inlineStr">
         <is>
-          <t>Mosa, Abu S</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="K28" s="14" t="n"/>
@@ -3752,7 +3752,7 @@
       <c r="N28" s="14" t="n"/>
       <c r="O28" s="14" t="inlineStr">
         <is>
-          <t>Osborne, John D</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="P28" s="14" t="n"/>
@@ -3761,7 +3761,7 @@
       <c r="S28" s="14" t="n"/>
       <c r="T28" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="U28" s="14" t="n"/>
@@ -3802,7 +3802,7 @@
       <c r="I29" s="14" t="n"/>
       <c r="J29" s="14" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Chong, Zechen</t>
         </is>
       </c>
       <c r="K29" s="14" t="n"/>
@@ -3820,7 +3820,7 @@
       <c r="S29" s="14" t="n"/>
       <c r="T29" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="U29" s="14" t="n"/>
@@ -3861,7 +3861,7 @@
       <c r="I30" s="14" t="n"/>
       <c r="J30" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="K30" s="14" t="n"/>
@@ -3870,7 +3870,7 @@
       <c r="N30" s="14" t="n"/>
       <c r="O30" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jin (Campus)</t>
+          <t>Osborne, John D</t>
         </is>
       </c>
       <c r="P30" s="14" t="n"/>
@@ -3918,7 +3918,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Osborne, John D</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
@@ -3928,7 +3928,7 @@
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reassign to three PI-safe reviewers per abstract; keep Lana cells.
- Add reassign_three_reviewers_pi_safe.py: cols 5/10/15 only, clear col 20,
  block own-lab reviewer per PI from Sheet0, preserve Garmire,Lana cells.
- Update workbook assignments accordingly.
- Document randomize_reviewers_keep_lana.py as legacy four-column path.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/ATTIS abstract submission_April 21, 2026_09.24_with_review_assignments.xlsx
+++ b/ATTIS abstract submission_April 21, 2026_09.24_with_review_assignments.xlsx
@@ -2208,7 +2208,7 @@
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>Osborne, John D</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="F2" s="14" t="n"/>
@@ -2217,7 +2217,7 @@
       <c r="I2" s="14" t="n"/>
       <c r="J2" s="14" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="K2" s="14" t="n"/>
@@ -2226,18 +2226,14 @@
       <c r="N2" s="14" t="n"/>
       <c r="O2" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jin (Campus)</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="P2" s="14" t="n"/>
       <c r="Q2" s="14" t="n"/>
       <c r="R2" s="14" t="n"/>
       <c r="S2" s="14" t="n"/>
-      <c r="T2" s="14" t="inlineStr">
-        <is>
-          <t>Mosa, Abu S</t>
-        </is>
-      </c>
+      <c r="T2" s="14" t="n"/>
       <c r="U2" s="14" t="n"/>
       <c r="V2" s="14" t="n"/>
       <c r="W2" s="14" t="n"/>
@@ -2267,7 +2263,7 @@
       </c>
       <c r="E3" s="14" t="inlineStr">
         <is>
-          <t>Osborne, John D</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="F3" s="14" t="n"/>
@@ -2276,7 +2272,7 @@
       <c r="I3" s="14" t="n"/>
       <c r="J3" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="K3" s="14" t="n"/>
@@ -2285,18 +2281,14 @@
       <c r="N3" s="14" t="n"/>
       <c r="O3" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="P3" s="14" t="n"/>
       <c r="Q3" s="14" t="n"/>
       <c r="R3" s="14" t="n"/>
       <c r="S3" s="14" t="n"/>
-      <c r="T3" s="14" t="inlineStr">
-        <is>
-          <t>Mosa, Abu S</t>
-        </is>
-      </c>
+      <c r="T3" s="14" t="n"/>
       <c r="U3" s="14" t="n"/>
       <c r="V3" s="14" t="n"/>
       <c r="W3" s="14" t="n"/>
@@ -2322,7 +2314,7 @@
       </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
-          <t>Mosa, Abu S</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="F4" s="14" t="n"/>
@@ -2331,7 +2323,7 @@
       <c r="I4" s="14" t="n"/>
       <c r="J4" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="K4" s="14" t="n"/>
@@ -2347,11 +2339,7 @@
       <c r="Q4" s="14" t="n"/>
       <c r="R4" s="14" t="n"/>
       <c r="S4" s="14" t="n"/>
-      <c r="T4" s="14" t="inlineStr">
-        <is>
-          <t>Jinzhuang Dou</t>
-        </is>
-      </c>
+      <c r="T4" s="14" t="n"/>
       <c r="U4" s="14" t="n"/>
       <c r="V4" s="14" t="n"/>
       <c r="W4" s="14" t="n"/>
@@ -2381,7 +2369,7 @@
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
-          <t>Amy Wang</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="F5" s="14" t="n"/>
@@ -2390,7 +2378,7 @@
       <c r="I5" s="14" t="n"/>
       <c r="J5" s="14" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="K5" s="14" t="n"/>
@@ -2399,18 +2387,14 @@
       <c r="N5" s="14" t="n"/>
       <c r="O5" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Osborne, John D</t>
         </is>
       </c>
       <c r="P5" s="14" t="n"/>
       <c r="Q5" s="14" t="n"/>
       <c r="R5" s="14" t="n"/>
       <c r="S5" s="14" t="n"/>
-      <c r="T5" s="14" t="inlineStr">
-        <is>
-          <t>Mosa, Abu S</t>
-        </is>
-      </c>
+      <c r="T5" s="14" t="n"/>
       <c r="U5" s="14" t="n"/>
       <c r="V5" s="14" t="n"/>
       <c r="W5" s="14" t="n"/>
@@ -2440,7 +2424,7 @@
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="F6" s="14" t="n"/>
@@ -2449,7 +2433,7 @@
       <c r="I6" s="14" t="n"/>
       <c r="J6" s="14" t="inlineStr">
         <is>
-          <t>Mosa, Abu S</t>
+          <t>Osborne, John D</t>
         </is>
       </c>
       <c r="K6" s="14" t="n"/>
@@ -2465,11 +2449,7 @@
       <c r="Q6" s="14" t="n"/>
       <c r="R6" s="14" t="n"/>
       <c r="S6" s="14" t="n"/>
-      <c r="T6" s="14" t="inlineStr">
-        <is>
-          <t>Chen, Jin (Campus)</t>
-        </is>
-      </c>
+      <c r="T6" s="14" t="n"/>
       <c r="U6" s="14" t="n"/>
       <c r="V6" s="14" t="n"/>
       <c r="W6" s="14" t="n"/>
@@ -2499,7 +2479,7 @@
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="F7" s="14" t="n"/>
@@ -2508,7 +2488,7 @@
       <c r="I7" s="14" t="n"/>
       <c r="J7" s="14" t="inlineStr">
         <is>
-          <t>Mosa, Abu S</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="K7" s="14" t="n"/>
@@ -2517,18 +2497,14 @@
       <c r="N7" s="14" t="n"/>
       <c r="O7" s="14" t="inlineStr">
         <is>
-          <t>Osborne, John D</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="P7" s="14" t="n"/>
       <c r="Q7" s="14" t="n"/>
       <c r="R7" s="14" t="n"/>
       <c r="S7" s="14" t="n"/>
-      <c r="T7" s="14" t="inlineStr">
-        <is>
-          <t>Chen, Jin (Campus)</t>
-        </is>
-      </c>
+      <c r="T7" s="14" t="n"/>
       <c r="U7" s="14" t="n"/>
       <c r="V7" s="14" t="n"/>
       <c r="W7" s="14" t="n"/>
@@ -2558,7 +2534,7 @@
       </c>
       <c r="E8" s="14" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="F8" s="14" t="n"/>
@@ -2567,7 +2543,7 @@
       <c r="I8" s="14" t="n"/>
       <c r="J8" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jin (Campus)</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="K8" s="14" t="n"/>
@@ -2576,18 +2552,14 @@
       <c r="N8" s="14" t="n"/>
       <c r="O8" s="14" t="inlineStr">
         <is>
-          <t>Mosa, Abu S</t>
+          <t>Osborne, John D</t>
         </is>
       </c>
       <c r="P8" s="14" t="n"/>
       <c r="Q8" s="14" t="n"/>
       <c r="R8" s="14" t="n"/>
       <c r="S8" s="14" t="n"/>
-      <c r="T8" s="14" t="inlineStr">
-        <is>
-          <t>Chong, Zechen</t>
-        </is>
-      </c>
+      <c r="T8" s="14" t="n"/>
       <c r="U8" s="14" t="n"/>
       <c r="V8" s="14" t="n"/>
       <c r="W8" s="14" t="n"/>
@@ -2617,7 +2589,7 @@
       </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
-          <t>Amy Wang</t>
+          <t>Osborne, John D</t>
         </is>
       </c>
       <c r="F9" s="14" t="n"/>
@@ -2626,7 +2598,7 @@
       <c r="I9" s="14" t="n"/>
       <c r="J9" s="14" t="inlineStr">
         <is>
-          <t>Mosa, Abu S</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="K9" s="14" t="n"/>
@@ -2635,18 +2607,14 @@
       <c r="N9" s="14" t="n"/>
       <c r="O9" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jin (Campus)</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="P9" s="14" t="n"/>
       <c r="Q9" s="14" t="n"/>
       <c r="R9" s="14" t="n"/>
       <c r="S9" s="14" t="n"/>
-      <c r="T9" s="14" t="inlineStr">
-        <is>
-          <t>Chen, Jake Y</t>
-        </is>
-      </c>
+      <c r="T9" s="14" t="n"/>
       <c r="U9" s="14" t="n"/>
       <c r="V9" s="14" t="n"/>
       <c r="W9" s="14" t="n"/>
@@ -2676,7 +2644,7 @@
       </c>
       <c r="E10" s="14" t="inlineStr">
         <is>
-          <t>Mosa, Abu S</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="F10" s="14" t="n"/>
@@ -2685,7 +2653,7 @@
       <c r="I10" s="14" t="n"/>
       <c r="J10" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="K10" s="14" t="n"/>
@@ -2694,18 +2662,14 @@
       <c r="N10" s="14" t="n"/>
       <c r="O10" s="14" t="inlineStr">
         <is>
-          <t>Amy Wang</t>
+          <t>Osborne, John D</t>
         </is>
       </c>
       <c r="P10" s="14" t="n"/>
       <c r="Q10" s="14" t="n"/>
       <c r="R10" s="14" t="n"/>
       <c r="S10" s="14" t="n"/>
-      <c r="T10" s="14" t="inlineStr">
-        <is>
-          <t>Chen, Jin (Campus)</t>
-        </is>
-      </c>
+      <c r="T10" s="14" t="n"/>
       <c r="U10" s="14" t="n"/>
       <c r="V10" s="14" t="n"/>
       <c r="W10" s="14" t="n"/>
@@ -2735,7 +2699,7 @@
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
-          <t>Amy Wang</t>
+          <t>Chong, Zechen</t>
         </is>
       </c>
       <c r="F11" s="14" t="n"/>
@@ -2744,7 +2708,7 @@
       <c r="I11" s="14" t="n"/>
       <c r="J11" s="14" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="K11" s="14" t="n"/>
@@ -2753,18 +2717,14 @@
       <c r="N11" s="14" t="n"/>
       <c r="O11" s="14" t="inlineStr">
         <is>
-          <t>Mosa, Abu S</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="P11" s="14" t="n"/>
       <c r="Q11" s="14" t="n"/>
       <c r="R11" s="14" t="n"/>
       <c r="S11" s="14" t="n"/>
-      <c r="T11" s="14" t="inlineStr">
-        <is>
-          <t>Chen, Jake Y</t>
-        </is>
-      </c>
+      <c r="T11" s="14" t="n"/>
       <c r="U11" s="14" t="n"/>
       <c r="V11" s="14" t="n"/>
       <c r="W11" s="14" t="n"/>
@@ -2790,7 +2750,7 @@
       </c>
       <c r="E12" s="14" t="inlineStr">
         <is>
-          <t>Mosa, Abu S</t>
+          <t>Osborne, John D</t>
         </is>
       </c>
       <c r="F12" s="14" t="n"/>
@@ -2808,18 +2768,14 @@
       <c r="N12" s="14" t="n"/>
       <c r="O12" s="14" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="P12" s="14" t="n"/>
       <c r="Q12" s="14" t="n"/>
       <c r="R12" s="14" t="n"/>
       <c r="S12" s="14" t="n"/>
-      <c r="T12" s="14" t="inlineStr">
-        <is>
-          <t>Chen, Jake Y</t>
-        </is>
-      </c>
+      <c r="T12" s="14" t="n"/>
       <c r="U12" s="14" t="n"/>
       <c r="V12" s="14" t="n"/>
       <c r="W12" s="14" t="n"/>
@@ -2849,7 +2805,7 @@
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jin (Campus)</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="F13" s="14" t="n"/>
@@ -2858,7 +2814,7 @@
       <c r="I13" s="14" t="n"/>
       <c r="J13" s="14" t="inlineStr">
         <is>
-          <t>Osborne, John D</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="K13" s="14" t="n"/>
@@ -2867,18 +2823,14 @@
       <c r="N13" s="14" t="n"/>
       <c r="O13" s="14" t="inlineStr">
         <is>
-          <t>Amy Wang</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="P13" s="14" t="n"/>
       <c r="Q13" s="14" t="n"/>
       <c r="R13" s="14" t="n"/>
       <c r="S13" s="14" t="n"/>
-      <c r="T13" s="14" t="inlineStr">
-        <is>
-          <t>Mosa, Abu S</t>
-        </is>
-      </c>
+      <c r="T13" s="14" t="n"/>
       <c r="U13" s="14" t="n"/>
       <c r="V13" s="14" t="n"/>
       <c r="W13" s="14" t="n"/>
@@ -2917,7 +2869,7 @@
       <c r="I14" s="14" t="n"/>
       <c r="J14" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="K14" s="14" t="n"/>
@@ -2926,18 +2878,14 @@
       <c r="N14" s="14" t="n"/>
       <c r="O14" s="14" t="inlineStr">
         <is>
-          <t>Amy Wang</t>
+          <t>Chong, Zechen</t>
         </is>
       </c>
       <c r="P14" s="14" t="n"/>
       <c r="Q14" s="14" t="n"/>
       <c r="R14" s="14" t="n"/>
       <c r="S14" s="14" t="n"/>
-      <c r="T14" s="14" t="inlineStr">
-        <is>
-          <t>Chen, Jake Y</t>
-        </is>
-      </c>
+      <c r="T14" s="14" t="n"/>
       <c r="U14" s="14" t="n"/>
       <c r="V14" s="14" t="n"/>
       <c r="W14" s="14" t="n"/>
@@ -2967,7 +2915,7 @@
       </c>
       <c r="E15" s="14" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Chong, Zechen</t>
         </is>
       </c>
       <c r="F15" s="14" t="n"/>
@@ -2992,11 +2940,7 @@
       <c r="Q15" s="14" t="n"/>
       <c r="R15" s="14" t="n"/>
       <c r="S15" s="14" t="n"/>
-      <c r="T15" s="14" t="inlineStr">
-        <is>
-          <t>Chong, Zechen</t>
-        </is>
-      </c>
+      <c r="T15" s="14" t="n"/>
       <c r="U15" s="14" t="n"/>
       <c r="V15" s="14" t="n"/>
       <c r="W15" s="14" t="n"/>
@@ -3035,7 +2979,7 @@
       <c r="I16" s="14" t="n"/>
       <c r="J16" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="K16" s="14" t="n"/>
@@ -3044,18 +2988,14 @@
       <c r="N16" s="14" t="n"/>
       <c r="O16" s="14" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="P16" s="14" t="n"/>
       <c r="Q16" s="14" t="n"/>
       <c r="R16" s="14" t="n"/>
       <c r="S16" s="14" t="n"/>
-      <c r="T16" s="14" t="inlineStr">
-        <is>
-          <t>Chen, Jake Y</t>
-        </is>
-      </c>
+      <c r="T16" s="14" t="n"/>
       <c r="U16" s="14" t="n"/>
       <c r="V16" s="14" t="n"/>
       <c r="W16" s="14" t="n"/>
@@ -3094,7 +3034,7 @@
       <c r="I17" s="14" t="n"/>
       <c r="J17" s="14" t="inlineStr">
         <is>
-          <t>Osborne, John D</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="K17" s="14" t="n"/>
@@ -3110,11 +3050,7 @@
       <c r="Q17" s="14" t="n"/>
       <c r="R17" s="14" t="n"/>
       <c r="S17" s="14" t="n"/>
-      <c r="T17" s="14" t="inlineStr">
-        <is>
-          <t>Amy Wang</t>
-        </is>
-      </c>
+      <c r="T17" s="14" t="n"/>
       <c r="U17" s="14" t="n"/>
       <c r="V17" s="14" t="n"/>
       <c r="W17" s="14" t="n"/>
@@ -3144,7 +3080,7 @@
       </c>
       <c r="E18" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="F18" s="14" t="n"/>
@@ -3153,7 +3089,7 @@
       <c r="I18" s="14" t="n"/>
       <c r="J18" s="14" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Chong, Zechen</t>
         </is>
       </c>
       <c r="K18" s="14" t="n"/>
@@ -3162,18 +3098,14 @@
       <c r="N18" s="14" t="n"/>
       <c r="O18" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="P18" s="14" t="n"/>
       <c r="Q18" s="14" t="n"/>
       <c r="R18" s="14" t="n"/>
       <c r="S18" s="14" t="n"/>
-      <c r="T18" s="14" t="inlineStr">
-        <is>
-          <t>Chen, Jin (Campus)</t>
-        </is>
-      </c>
+      <c r="T18" s="14" t="n"/>
       <c r="U18" s="14" t="n"/>
       <c r="V18" s="14" t="n"/>
       <c r="W18" s="14" t="n"/>
@@ -3203,7 +3135,7 @@
       </c>
       <c r="E19" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="F19" s="14" t="n"/>
@@ -3221,18 +3153,14 @@
       <c r="N19" s="14" t="n"/>
       <c r="O19" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Chong, Zechen</t>
         </is>
       </c>
       <c r="P19" s="14" t="n"/>
       <c r="Q19" s="14" t="n"/>
       <c r="R19" s="14" t="n"/>
       <c r="S19" s="14" t="n"/>
-      <c r="T19" s="14" t="inlineStr">
-        <is>
-          <t>Jinzhuang Dou</t>
-        </is>
-      </c>
+      <c r="T19" s="14" t="n"/>
       <c r="U19" s="14" t="n"/>
       <c r="V19" s="14" t="n"/>
       <c r="W19" s="14" t="n"/>
@@ -3262,7 +3190,7 @@
       </c>
       <c r="E20" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="F20" s="14" t="n"/>
@@ -3271,7 +3199,7 @@
       <c r="I20" s="14" t="n"/>
       <c r="J20" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="K20" s="14" t="n"/>
@@ -3280,18 +3208,14 @@
       <c r="N20" s="14" t="n"/>
       <c r="O20" s="14" t="inlineStr">
         <is>
-          <t>Amy Wang</t>
+          <t>Chong, Zechen</t>
         </is>
       </c>
       <c r="P20" s="14" t="n"/>
       <c r="Q20" s="14" t="n"/>
       <c r="R20" s="14" t="n"/>
       <c r="S20" s="14" t="n"/>
-      <c r="T20" s="14" t="inlineStr">
-        <is>
-          <t>Jinzhuang Dou</t>
-        </is>
-      </c>
+      <c r="T20" s="14" t="n"/>
       <c r="U20" s="14" t="n"/>
       <c r="V20" s="14" t="n"/>
       <c r="W20" s="14" t="n"/>
@@ -3330,7 +3254,7 @@
       <c r="I21" s="14" t="n"/>
       <c r="J21" s="14" t="inlineStr">
         <is>
-          <t>Amy Wang</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="K21" s="14" t="n"/>
@@ -3339,18 +3263,14 @@
       <c r="N21" s="14" t="n"/>
       <c r="O21" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="P21" s="14" t="n"/>
       <c r="Q21" s="14" t="n"/>
       <c r="R21" s="14" t="n"/>
       <c r="S21" s="14" t="n"/>
-      <c r="T21" s="14" t="inlineStr">
-        <is>
-          <t>Osborne, John D</t>
-        </is>
-      </c>
+      <c r="T21" s="14" t="n"/>
       <c r="U21" s="14" t="n"/>
       <c r="V21" s="14" t="n"/>
       <c r="W21" s="14" t="n"/>
@@ -3380,7 +3300,7 @@
       </c>
       <c r="E22" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jin (Campus)</t>
+          <t>Osborne, John D</t>
         </is>
       </c>
       <c r="F22" s="14" t="n"/>
@@ -3389,7 +3309,7 @@
       <c r="I22" s="14" t="n"/>
       <c r="J22" s="14" t="inlineStr">
         <is>
-          <t>Osborne, John D</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="K22" s="14" t="n"/>
@@ -3398,18 +3318,14 @@
       <c r="N22" s="14" t="n"/>
       <c r="O22" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Chong, Zechen</t>
         </is>
       </c>
       <c r="P22" s="14" t="n"/>
       <c r="Q22" s="14" t="n"/>
       <c r="R22" s="14" t="n"/>
       <c r="S22" s="14" t="n"/>
-      <c r="T22" s="14" t="inlineStr">
-        <is>
-          <t>Mosa, Abu S</t>
-        </is>
-      </c>
+      <c r="T22" s="14" t="n"/>
       <c r="U22" s="14" t="n"/>
       <c r="V22" s="14" t="n"/>
       <c r="W22" s="14" t="n"/>
@@ -3464,11 +3380,7 @@
       <c r="Q23" s="14" t="n"/>
       <c r="R23" s="14" t="n"/>
       <c r="S23" s="14" t="n"/>
-      <c r="T23" s="14" t="inlineStr">
-        <is>
-          <t>Mosa, Abu S</t>
-        </is>
-      </c>
+      <c r="T23" s="14" t="n"/>
       <c r="U23" s="14" t="n"/>
       <c r="V23" s="14" t="n"/>
       <c r="W23" s="14" t="n"/>
@@ -3516,18 +3428,14 @@
       <c r="N24" s="14" t="n"/>
       <c r="O24" s="14" t="inlineStr">
         <is>
-          <t>Amy Wang</t>
+          <t>Chong, Zechen</t>
         </is>
       </c>
       <c r="P24" s="14" t="n"/>
       <c r="Q24" s="14" t="n"/>
       <c r="R24" s="14" t="n"/>
       <c r="S24" s="14" t="n"/>
-      <c r="T24" s="14" t="inlineStr">
-        <is>
-          <t>Mosa, Abu S</t>
-        </is>
-      </c>
+      <c r="T24" s="14" t="n"/>
       <c r="U24" s="14" t="n"/>
       <c r="V24" s="14" t="n"/>
       <c r="W24" s="14" t="n"/>
@@ -3566,7 +3474,7 @@
       <c r="I25" s="14" t="n"/>
       <c r="J25" s="14" t="inlineStr">
         <is>
-          <t>Amy Wang</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="K25" s="14" t="n"/>
@@ -3575,18 +3483,14 @@
       <c r="N25" s="14" t="n"/>
       <c r="O25" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="P25" s="14" t="n"/>
       <c r="Q25" s="14" t="n"/>
       <c r="R25" s="14" t="n"/>
       <c r="S25" s="14" t="n"/>
-      <c r="T25" s="14" t="inlineStr">
-        <is>
-          <t>Mosa, Abu S</t>
-        </is>
-      </c>
+      <c r="T25" s="14" t="n"/>
       <c r="U25" s="14" t="n"/>
       <c r="V25" s="14" t="n"/>
       <c r="W25" s="14" t="n"/>
@@ -3625,7 +3529,7 @@
       <c r="I26" s="14" t="n"/>
       <c r="J26" s="14" t="inlineStr">
         <is>
-          <t>Mosa, Abu S</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="K26" s="14" t="n"/>
@@ -3634,18 +3538,14 @@
       <c r="N26" s="14" t="n"/>
       <c r="O26" s="14" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="P26" s="14" t="n"/>
       <c r="Q26" s="14" t="n"/>
       <c r="R26" s="14" t="n"/>
       <c r="S26" s="14" t="n"/>
-      <c r="T26" s="14" t="inlineStr">
-        <is>
-          <t>Chen, Jin (Campus)</t>
-        </is>
-      </c>
+      <c r="T26" s="14" t="n"/>
       <c r="U26" s="14" t="n"/>
       <c r="V26" s="14" t="n"/>
       <c r="W26" s="14" t="n"/>
@@ -3684,7 +3584,7 @@
       <c r="I27" s="14" t="n"/>
       <c r="J27" s="14" t="inlineStr">
         <is>
-          <t>Amy Wang</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="K27" s="14" t="n"/>
@@ -3693,18 +3593,14 @@
       <c r="N27" s="14" t="n"/>
       <c r="O27" s="14" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="P27" s="14" t="n"/>
       <c r="Q27" s="14" t="n"/>
       <c r="R27" s="14" t="n"/>
       <c r="S27" s="14" t="n"/>
-      <c r="T27" s="14" t="inlineStr">
-        <is>
-          <t>Chong, Zechen</t>
-        </is>
-      </c>
+      <c r="T27" s="14" t="n"/>
       <c r="U27" s="14" t="n"/>
       <c r="V27" s="14" t="n"/>
       <c r="W27" s="14" t="n"/>
@@ -3743,7 +3639,7 @@
       <c r="I28" s="14" t="n"/>
       <c r="J28" s="14" t="inlineStr">
         <is>
-          <t>Amy Wang</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="K28" s="14" t="n"/>
@@ -3752,18 +3648,14 @@
       <c r="N28" s="14" t="n"/>
       <c r="O28" s="14" t="inlineStr">
         <is>
-          <t>Mosa, Abu S</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="P28" s="14" t="n"/>
       <c r="Q28" s="14" t="n"/>
       <c r="R28" s="14" t="n"/>
       <c r="S28" s="14" t="n"/>
-      <c r="T28" s="14" t="inlineStr">
-        <is>
-          <t>Chen, Jin (Campus)</t>
-        </is>
-      </c>
+      <c r="T28" s="14" t="n"/>
       <c r="U28" s="14" t="n"/>
       <c r="V28" s="14" t="n"/>
       <c r="W28" s="14" t="n"/>
@@ -3818,11 +3710,7 @@
       <c r="Q29" s="14" t="n"/>
       <c r="R29" s="14" t="n"/>
       <c r="S29" s="14" t="n"/>
-      <c r="T29" s="14" t="inlineStr">
-        <is>
-          <t>Chen, Jake Y</t>
-        </is>
-      </c>
+      <c r="T29" s="14" t="n"/>
       <c r="U29" s="14" t="n"/>
       <c r="V29" s="14" t="n"/>
       <c r="W29" s="14" t="n"/>
@@ -3852,7 +3740,7 @@
       </c>
       <c r="E30" s="14" t="inlineStr">
         <is>
-          <t>Amy Wang</t>
+          <t>Chong, Zechen</t>
         </is>
       </c>
       <c r="F30" s="14" t="n"/>
@@ -3870,18 +3758,14 @@
       <c r="N30" s="14" t="n"/>
       <c r="O30" s="14" t="inlineStr">
         <is>
-          <t>Osborne, John D</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="P30" s="14" t="n"/>
       <c r="Q30" s="14" t="n"/>
       <c r="R30" s="14" t="n"/>
       <c r="S30" s="14" t="n"/>
-      <c r="T30" s="14" t="inlineStr">
-        <is>
-          <t>Chong, Zechen</t>
-        </is>
-      </c>
+      <c r="T30" s="14" t="n"/>
       <c r="U30" s="14" t="n"/>
       <c r="V30" s="14" t="n"/>
       <c r="W30" s="14" t="n"/>
@@ -3918,17 +3802,12 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
-        </is>
-      </c>
-      <c r="T31" t="inlineStr">
-        <is>
-          <t>Mosa, Abu S</t>
+          <t>Amy Wang</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Balance non-Lana reviewer loads to 11 each; keep Lana fixes
Add balance_reviewer_loads_keep_lana.py (greedy + local search).
Preserved Garmire,Lana cells; PI rules unchanged; col20 cleared.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/ATTIS abstract submission_April 21, 2026_09.24_with_review_assignments.xlsx
+++ b/ATTIS abstract submission_April 21, 2026_09.24_with_review_assignments.xlsx
@@ -2208,7 +2208,7 @@
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="F2" s="14" t="n"/>
@@ -2217,7 +2217,7 @@
       <c r="I2" s="14" t="n"/>
       <c r="J2" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Chong, Zechen</t>
         </is>
       </c>
       <c r="K2" s="14" t="n"/>
@@ -2226,7 +2226,7 @@
       <c r="N2" s="14" t="n"/>
       <c r="O2" s="14" t="inlineStr">
         <is>
-          <t>Amy Wang</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="P2" s="14" t="n"/>
@@ -2263,7 +2263,7 @@
       </c>
       <c r="E3" s="14" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Chong, Zechen</t>
         </is>
       </c>
       <c r="F3" s="14" t="n"/>
@@ -2272,7 +2272,7 @@
       <c r="I3" s="14" t="n"/>
       <c r="J3" s="14" t="inlineStr">
         <is>
-          <t>Mosa, Abu S</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="K3" s="14" t="n"/>
@@ -2281,7 +2281,7 @@
       <c r="N3" s="14" t="n"/>
       <c r="O3" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jin (Campus)</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="P3" s="14" t="n"/>
@@ -2323,7 +2323,7 @@
       <c r="I4" s="14" t="n"/>
       <c r="J4" s="14" t="inlineStr">
         <is>
-          <t>Amy Wang</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="K4" s="14" t="n"/>
@@ -2369,7 +2369,7 @@
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Osborne, John D</t>
         </is>
       </c>
       <c r="F5" s="14" t="n"/>
@@ -2378,7 +2378,7 @@
       <c r="I5" s="14" t="n"/>
       <c r="J5" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="K5" s="14" t="n"/>
@@ -2387,7 +2387,7 @@
       <c r="N5" s="14" t="n"/>
       <c r="O5" s="14" t="inlineStr">
         <is>
-          <t>Osborne, John D</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="P5" s="14" t="n"/>
@@ -2424,7 +2424,7 @@
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="F6" s="14" t="n"/>
@@ -2433,7 +2433,7 @@
       <c r="I6" s="14" t="n"/>
       <c r="J6" s="14" t="inlineStr">
         <is>
-          <t>Osborne, John D</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="K6" s="14" t="n"/>
@@ -2442,7 +2442,7 @@
       <c r="N6" s="14" t="n"/>
       <c r="O6" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="P6" s="14" t="n"/>
@@ -2479,7 +2479,7 @@
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="F7" s="14" t="n"/>
@@ -2488,7 +2488,7 @@
       <c r="I7" s="14" t="n"/>
       <c r="J7" s="14" t="inlineStr">
         <is>
-          <t>Amy Wang</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="K7" s="14" t="n"/>
@@ -2497,7 +2497,7 @@
       <c r="N7" s="14" t="n"/>
       <c r="O7" s="14" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="P7" s="14" t="n"/>
@@ -2534,7 +2534,7 @@
       </c>
       <c r="E8" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jin (Campus)</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="F8" s="14" t="n"/>
@@ -2543,7 +2543,7 @@
       <c r="I8" s="14" t="n"/>
       <c r="J8" s="14" t="inlineStr">
         <is>
-          <t>Amy Wang</t>
+          <t>Osborne, John D</t>
         </is>
       </c>
       <c r="K8" s="14" t="n"/>
@@ -2552,7 +2552,7 @@
       <c r="N8" s="14" t="n"/>
       <c r="O8" s="14" t="inlineStr">
         <is>
-          <t>Osborne, John D</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="P8" s="14" t="n"/>
@@ -2589,7 +2589,7 @@
       </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
-          <t>Osborne, John D</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="F9" s="14" t="n"/>
@@ -2598,7 +2598,7 @@
       <c r="I9" s="14" t="n"/>
       <c r="J9" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="K9" s="14" t="n"/>
@@ -2607,7 +2607,7 @@
       <c r="N9" s="14" t="n"/>
       <c r="O9" s="14" t="inlineStr">
         <is>
-          <t>Amy Wang</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="P9" s="14" t="n"/>
@@ -2644,7 +2644,7 @@
       </c>
       <c r="E10" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jin (Campus)</t>
+          <t>Chong, Zechen</t>
         </is>
       </c>
       <c r="F10" s="14" t="n"/>
@@ -2662,7 +2662,7 @@
       <c r="N10" s="14" t="n"/>
       <c r="O10" s="14" t="inlineStr">
         <is>
-          <t>Osborne, John D</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="P10" s="14" t="n"/>
@@ -2708,7 +2708,7 @@
       <c r="I11" s="14" t="n"/>
       <c r="J11" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jin (Campus)</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="K11" s="14" t="n"/>
@@ -2717,7 +2717,7 @@
       <c r="N11" s="14" t="n"/>
       <c r="O11" s="14" t="inlineStr">
         <is>
-          <t>Amy Wang</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="P11" s="14" t="n"/>
@@ -2750,7 +2750,7 @@
       </c>
       <c r="E12" s="14" t="inlineStr">
         <is>
-          <t>Osborne, John D</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="F12" s="14" t="n"/>
@@ -2768,7 +2768,7 @@
       <c r="N12" s="14" t="n"/>
       <c r="O12" s="14" t="inlineStr">
         <is>
-          <t>Mosa, Abu S</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="P12" s="14" t="n"/>
@@ -2814,7 +2814,7 @@
       <c r="I13" s="14" t="n"/>
       <c r="J13" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="K13" s="14" t="n"/>
@@ -2878,7 +2878,7 @@
       <c r="N14" s="14" t="n"/>
       <c r="O14" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="P14" s="14" t="n"/>
@@ -2915,7 +2915,7 @@
       </c>
       <c r="E15" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Osborne, John D</t>
         </is>
       </c>
       <c r="F15" s="14" t="n"/>
@@ -2979,7 +2979,7 @@
       <c r="I16" s="14" t="n"/>
       <c r="J16" s="14" t="inlineStr">
         <is>
-          <t>Amy Wang</t>
+          <t>Chong, Zechen</t>
         </is>
       </c>
       <c r="K16" s="14" t="n"/>
@@ -3025,7 +3025,7 @@
       </c>
       <c r="E17" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="F17" s="14" t="n"/>
@@ -3034,7 +3034,7 @@
       <c r="I17" s="14" t="n"/>
       <c r="J17" s="14" t="inlineStr">
         <is>
-          <t>Amy Wang</t>
+          <t>Osborne, John D</t>
         </is>
       </c>
       <c r="K17" s="14" t="n"/>
@@ -3080,7 +3080,7 @@
       </c>
       <c r="E18" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="F18" s="14" t="n"/>
@@ -3089,7 +3089,7 @@
       <c r="I18" s="14" t="n"/>
       <c r="J18" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="K18" s="14" t="n"/>
@@ -3098,7 +3098,7 @@
       <c r="N18" s="14" t="n"/>
       <c r="O18" s="14" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Osborne, John D</t>
         </is>
       </c>
       <c r="P18" s="14" t="n"/>
@@ -3135,7 +3135,7 @@
       </c>
       <c r="E19" s="14" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Chong, Zechen</t>
         </is>
       </c>
       <c r="F19" s="14" t="n"/>
@@ -3153,7 +3153,7 @@
       <c r="N19" s="14" t="n"/>
       <c r="O19" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="P19" s="14" t="n"/>
@@ -3190,7 +3190,7 @@
       </c>
       <c r="E20" s="14" t="inlineStr">
         <is>
-          <t>Amy Wang</t>
+          <t>Osborne, John D</t>
         </is>
       </c>
       <c r="F20" s="14" t="n"/>
@@ -3199,7 +3199,7 @@
       <c r="I20" s="14" t="n"/>
       <c r="J20" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="K20" s="14" t="n"/>
@@ -3300,7 +3300,7 @@
       </c>
       <c r="E22" s="14" t="inlineStr">
         <is>
-          <t>Osborne, John D</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="F22" s="14" t="n"/>
@@ -3309,7 +3309,7 @@
       <c r="I22" s="14" t="n"/>
       <c r="J22" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jin (Campus)</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="K22" s="14" t="n"/>
@@ -3318,7 +3318,7 @@
       <c r="N22" s="14" t="n"/>
       <c r="O22" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="P22" s="14" t="n"/>
@@ -3364,7 +3364,7 @@
       <c r="I23" s="14" t="n"/>
       <c r="J23" s="14" t="inlineStr">
         <is>
-          <t>Amy Wang</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="K23" s="14" t="n"/>
@@ -3373,7 +3373,7 @@
       <c r="N23" s="14" t="n"/>
       <c r="O23" s="14" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="P23" s="14" t="n"/>
@@ -3419,7 +3419,7 @@
       <c r="I24" s="14" t="n"/>
       <c r="J24" s="14" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Osborne, John D</t>
         </is>
       </c>
       <c r="K24" s="14" t="n"/>
@@ -3428,7 +3428,7 @@
       <c r="N24" s="14" t="n"/>
       <c r="O24" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="P24" s="14" t="n"/>
@@ -3465,7 +3465,7 @@
       </c>
       <c r="E25" s="14" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="F25" s="14" t="n"/>
@@ -3474,7 +3474,7 @@
       <c r="I25" s="14" t="n"/>
       <c r="J25" s="14" t="inlineStr">
         <is>
-          <t>Mosa, Abu S</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="K25" s="14" t="n"/>
@@ -3529,7 +3529,7 @@
       <c r="I26" s="14" t="n"/>
       <c r="J26" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="K26" s="14" t="n"/>
@@ -3538,7 +3538,7 @@
       <c r="N26" s="14" t="n"/>
       <c r="O26" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jin (Campus)</t>
+          <t>Osborne, John D</t>
         </is>
       </c>
       <c r="P26" s="14" t="n"/>
@@ -3584,7 +3584,7 @@
       <c r="I27" s="14" t="n"/>
       <c r="J27" s="14" t="inlineStr">
         <is>
-          <t>Mosa, Abu S</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="K27" s="14" t="n"/>
@@ -3593,7 +3593,7 @@
       <c r="N27" s="14" t="n"/>
       <c r="O27" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Osborne, John D</t>
         </is>
       </c>
       <c r="P27" s="14" t="n"/>
@@ -3639,7 +3639,7 @@
       <c r="I28" s="14" t="n"/>
       <c r="J28" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jin (Campus)</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="K28" s="14" t="n"/>
@@ -3648,7 +3648,7 @@
       <c r="N28" s="14" t="n"/>
       <c r="O28" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Osborne, John D</t>
         </is>
       </c>
       <c r="P28" s="14" t="n"/>
@@ -3694,7 +3694,7 @@
       <c r="I29" s="14" t="n"/>
       <c r="J29" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="K29" s="14" t="n"/>
@@ -3703,7 +3703,7 @@
       <c r="N29" s="14" t="n"/>
       <c r="O29" s="14" t="inlineStr">
         <is>
-          <t>Mosa, Abu S</t>
+          <t>Chong, Zechen</t>
         </is>
       </c>
       <c r="P29" s="14" t="n"/>
@@ -3749,7 +3749,7 @@
       <c r="I30" s="14" t="n"/>
       <c r="J30" s="14" t="inlineStr">
         <is>
-          <t>Mosa, Abu S</t>
+          <t>Osborne, John D</t>
         </is>
       </c>
       <c r="K30" s="14" t="n"/>
@@ -3758,7 +3758,7 @@
       <c r="N30" s="14" t="n"/>
       <c r="O30" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jin (Campus)</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="P30" s="14" t="n"/>
@@ -3802,12 +3802,12 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Mosa, Abu S</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>Amy Wang</t>
+          <t>Chong, Zechen</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Balance loads in band 10–12 per reviewer (vs fixed 11)
Tunable LOAD_MIN/LOAD_MAX; multiset targets summing to flex slots.
Greedy by combination + faster local search (early exit when optimal).

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/ATTIS abstract submission_April 21, 2026_09.24_with_review_assignments.xlsx
+++ b/ATTIS abstract submission_April 21, 2026_09.24_with_review_assignments.xlsx
@@ -2208,7 +2208,7 @@
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="F2" s="14" t="n"/>
@@ -2217,7 +2217,7 @@
       <c r="I2" s="14" t="n"/>
       <c r="J2" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="K2" s="14" t="n"/>
@@ -2226,7 +2226,7 @@
       <c r="N2" s="14" t="n"/>
       <c r="O2" s="14" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Chong, Zechen</t>
         </is>
       </c>
       <c r="P2" s="14" t="n"/>
@@ -2263,7 +2263,7 @@
       </c>
       <c r="E3" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="F3" s="14" t="n"/>
@@ -2281,7 +2281,7 @@
       <c r="N3" s="14" t="n"/>
       <c r="O3" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="P3" s="14" t="n"/>
@@ -2323,7 +2323,7 @@
       <c r="I4" s="14" t="n"/>
       <c r="J4" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="K4" s="14" t="n"/>
@@ -2369,7 +2369,7 @@
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
-          <t>Osborne, John D</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="F5" s="14" t="n"/>
@@ -2378,7 +2378,7 @@
       <c r="I5" s="14" t="n"/>
       <c r="J5" s="14" t="inlineStr">
         <is>
-          <t>Mosa, Abu S</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="K5" s="14" t="n"/>
@@ -2387,7 +2387,7 @@
       <c r="N5" s="14" t="n"/>
       <c r="O5" s="14" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Osborne, John D</t>
         </is>
       </c>
       <c r="P5" s="14" t="n"/>
@@ -2424,7 +2424,7 @@
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
-          <t>Amy Wang</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="F6" s="14" t="n"/>
@@ -2433,7 +2433,7 @@
       <c r="I6" s="14" t="n"/>
       <c r="J6" s="14" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Chong, Zechen</t>
         </is>
       </c>
       <c r="K6" s="14" t="n"/>
@@ -2442,7 +2442,7 @@
       <c r="N6" s="14" t="n"/>
       <c r="O6" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Osborne, John D</t>
         </is>
       </c>
       <c r="P6" s="14" t="n"/>
@@ -2479,7 +2479,7 @@
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
-          <t>Amy Wang</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="F7" s="14" t="n"/>
@@ -2488,7 +2488,7 @@
       <c r="I7" s="14" t="n"/>
       <c r="J7" s="14" t="inlineStr">
         <is>
-          <t>Mosa, Abu S</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="K7" s="14" t="n"/>
@@ -2497,7 +2497,7 @@
       <c r="N7" s="14" t="n"/>
       <c r="O7" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jin (Campus)</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="P7" s="14" t="n"/>
@@ -2543,7 +2543,7 @@
       <c r="I8" s="14" t="n"/>
       <c r="J8" s="14" t="inlineStr">
         <is>
-          <t>Osborne, John D</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="K8" s="14" t="n"/>
@@ -2598,7 +2598,7 @@
       <c r="I9" s="14" t="n"/>
       <c r="J9" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jin (Campus)</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="K9" s="14" t="n"/>
@@ -2644,7 +2644,7 @@
       </c>
       <c r="E10" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="F10" s="14" t="n"/>
@@ -2699,7 +2699,7 @@
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="F11" s="14" t="n"/>
@@ -2708,7 +2708,7 @@
       <c r="I11" s="14" t="n"/>
       <c r="J11" s="14" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Chong, Zechen</t>
         </is>
       </c>
       <c r="K11" s="14" t="n"/>
@@ -2717,7 +2717,7 @@
       <c r="N11" s="14" t="n"/>
       <c r="O11" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="P11" s="14" t="n"/>
@@ -2750,7 +2750,7 @@
       </c>
       <c r="E12" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="F12" s="14" t="n"/>
@@ -2768,7 +2768,7 @@
       <c r="N12" s="14" t="n"/>
       <c r="O12" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jin (Campus)</t>
+          <t>Osborne, John D</t>
         </is>
       </c>
       <c r="P12" s="14" t="n"/>
@@ -2814,7 +2814,7 @@
       <c r="I13" s="14" t="n"/>
       <c r="J13" s="14" t="inlineStr">
         <is>
-          <t>Mosa, Abu S</t>
+          <t>Chong, Zechen</t>
         </is>
       </c>
       <c r="K13" s="14" t="n"/>
@@ -2823,7 +2823,7 @@
       <c r="N13" s="14" t="n"/>
       <c r="O13" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jin (Campus)</t>
+          <t>Osborne, John D</t>
         </is>
       </c>
       <c r="P13" s="14" t="n"/>
@@ -2915,7 +2915,7 @@
       </c>
       <c r="E15" s="14" t="inlineStr">
         <is>
-          <t>Osborne, John D</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="F15" s="14" t="n"/>
@@ -2933,7 +2933,7 @@
       <c r="N15" s="14" t="n"/>
       <c r="O15" s="14" t="inlineStr">
         <is>
-          <t>Amy Wang</t>
+          <t>Chong, Zechen</t>
         </is>
       </c>
       <c r="P15" s="14" t="n"/>
@@ -2970,7 +2970,7 @@
       </c>
       <c r="E16" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jin (Campus)</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="F16" s="14" t="n"/>
@@ -2979,7 +2979,7 @@
       <c r="I16" s="14" t="n"/>
       <c r="J16" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="K16" s="14" t="n"/>
@@ -2988,7 +2988,7 @@
       <c r="N16" s="14" t="n"/>
       <c r="O16" s="14" t="inlineStr">
         <is>
-          <t>Mosa, Abu S</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="P16" s="14" t="n"/>
@@ -3025,7 +3025,7 @@
       </c>
       <c r="E17" s="14" t="inlineStr">
         <is>
-          <t>Mosa, Abu S</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="F17" s="14" t="n"/>
@@ -3034,7 +3034,7 @@
       <c r="I17" s="14" t="n"/>
       <c r="J17" s="14" t="inlineStr">
         <is>
-          <t>Osborne, John D</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="K17" s="14" t="n"/>
@@ -3043,7 +3043,7 @@
       <c r="N17" s="14" t="n"/>
       <c r="O17" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="P17" s="14" t="n"/>
@@ -3089,7 +3089,7 @@
       <c r="I18" s="14" t="n"/>
       <c r="J18" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="K18" s="14" t="n"/>
@@ -3135,7 +3135,7 @@
       </c>
       <c r="E19" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="F19" s="14" t="n"/>
@@ -3153,7 +3153,7 @@
       <c r="N19" s="14" t="n"/>
       <c r="O19" s="14" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="P19" s="14" t="n"/>
@@ -3190,7 +3190,7 @@
       </c>
       <c r="E20" s="14" t="inlineStr">
         <is>
-          <t>Osborne, John D</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="F20" s="14" t="n"/>
@@ -3199,7 +3199,7 @@
       <c r="I20" s="14" t="n"/>
       <c r="J20" s="14" t="inlineStr">
         <is>
-          <t>Amy Wang</t>
+          <t>Chong, Zechen</t>
         </is>
       </c>
       <c r="K20" s="14" t="n"/>
@@ -3208,7 +3208,7 @@
       <c r="N20" s="14" t="n"/>
       <c r="O20" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="P20" s="14" t="n"/>
@@ -3254,7 +3254,7 @@
       <c r="I21" s="14" t="n"/>
       <c r="J21" s="14" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Chong, Zechen</t>
         </is>
       </c>
       <c r="K21" s="14" t="n"/>
@@ -3263,7 +3263,7 @@
       <c r="N21" s="14" t="n"/>
       <c r="O21" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jin (Campus)</t>
+          <t>Osborne, John D</t>
         </is>
       </c>
       <c r="P21" s="14" t="n"/>
@@ -3300,7 +3300,7 @@
       </c>
       <c r="E22" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jin (Campus)</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="F22" s="14" t="n"/>
@@ -3309,7 +3309,7 @@
       <c r="I22" s="14" t="n"/>
       <c r="J22" s="14" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Chong, Zechen</t>
         </is>
       </c>
       <c r="K22" s="14" t="n"/>
@@ -3318,7 +3318,7 @@
       <c r="N22" s="14" t="n"/>
       <c r="O22" s="14" t="inlineStr">
         <is>
-          <t>Amy Wang</t>
+          <t>Osborne, John D</t>
         </is>
       </c>
       <c r="P22" s="14" t="n"/>
@@ -3364,7 +3364,7 @@
       <c r="I23" s="14" t="n"/>
       <c r="J23" s="14" t="inlineStr">
         <is>
-          <t>Mosa, Abu S</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="K23" s="14" t="n"/>
@@ -3373,7 +3373,7 @@
       <c r="N23" s="14" t="n"/>
       <c r="O23" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="P23" s="14" t="n"/>
@@ -3419,7 +3419,7 @@
       <c r="I24" s="14" t="n"/>
       <c r="J24" s="14" t="inlineStr">
         <is>
-          <t>Osborne, John D</t>
+          <t>Chong, Zechen</t>
         </is>
       </c>
       <c r="K24" s="14" t="n"/>
@@ -3428,7 +3428,7 @@
       <c r="N24" s="14" t="n"/>
       <c r="O24" s="14" t="inlineStr">
         <is>
-          <t>Amy Wang</t>
+          <t>Osborne, John D</t>
         </is>
       </c>
       <c r="P24" s="14" t="n"/>
@@ -3465,7 +3465,7 @@
       </c>
       <c r="E25" s="14" t="inlineStr">
         <is>
-          <t>Mosa, Abu S</t>
+          <t>Chong, Zechen</t>
         </is>
       </c>
       <c r="F25" s="14" t="n"/>
@@ -3483,7 +3483,7 @@
       <c r="N25" s="14" t="n"/>
       <c r="O25" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jin (Campus)</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="P25" s="14" t="n"/>
@@ -3529,7 +3529,7 @@
       <c r="I26" s="14" t="n"/>
       <c r="J26" s="14" t="inlineStr">
         <is>
-          <t>Amy Wang</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="K26" s="14" t="n"/>
@@ -3538,7 +3538,7 @@
       <c r="N26" s="14" t="n"/>
       <c r="O26" s="14" t="inlineStr">
         <is>
-          <t>Osborne, John D</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="P26" s="14" t="n"/>
@@ -3584,7 +3584,7 @@
       <c r="I27" s="14" t="n"/>
       <c r="J27" s="14" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="K27" s="14" t="n"/>
@@ -3639,7 +3639,7 @@
       <c r="I28" s="14" t="n"/>
       <c r="J28" s="14" t="inlineStr">
         <is>
-          <t>Mosa, Abu S</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="K28" s="14" t="n"/>
@@ -3694,7 +3694,7 @@
       <c r="I29" s="14" t="n"/>
       <c r="J29" s="14" t="inlineStr">
         <is>
-          <t>Amy Wang</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="K29" s="14" t="n"/>
@@ -3703,7 +3703,7 @@
       <c r="N29" s="14" t="n"/>
       <c r="O29" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="P29" s="14" t="n"/>
@@ -3740,7 +3740,7 @@
       </c>
       <c r="E30" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="F30" s="14" t="n"/>
@@ -3749,7 +3749,7 @@
       <c r="I30" s="14" t="n"/>
       <c r="J30" s="14" t="inlineStr">
         <is>
-          <t>Osborne, John D</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="K30" s="14" t="n"/>
@@ -3758,7 +3758,7 @@
       <c r="N30" s="14" t="n"/>
       <c r="O30" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="P30" s="14" t="n"/>
@@ -3807,7 +3807,7 @@
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sync review assignment workbook with local copy
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/ATTIS abstract submission_April 21, 2026_09.24_with_review_assignments.xlsx
+++ b/ATTIS abstract submission_April 21, 2026_09.24_with_review_assignments.xlsx
@@ -2226,7 +2226,7 @@
       <c r="N2" s="14" t="n"/>
       <c r="O2" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="P2" s="14" t="n"/>
@@ -2263,7 +2263,7 @@
       </c>
       <c r="E3" s="14" t="inlineStr">
         <is>
-          <t>Amy Wang</t>
+          <t>Osborne, John D</t>
         </is>
       </c>
       <c r="F3" s="14" t="n"/>
@@ -2272,7 +2272,7 @@
       <c r="I3" s="14" t="n"/>
       <c r="J3" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jin (Campus)</t>
+          <t>Chong, Zechen</t>
         </is>
       </c>
       <c r="K3" s="14" t="n"/>
@@ -2281,7 +2281,7 @@
       <c r="N3" s="14" t="n"/>
       <c r="O3" s="14" t="inlineStr">
         <is>
-          <t>Mosa, Abu S</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="P3" s="14" t="n"/>
@@ -2314,7 +2314,7 @@
       </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jin (Campus)</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="F4" s="14" t="n"/>
@@ -2323,7 +2323,7 @@
       <c r="I4" s="14" t="n"/>
       <c r="J4" s="14" t="inlineStr">
         <is>
-          <t>Mosa, Abu S</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="K4" s="14" t="n"/>
@@ -2387,7 +2387,7 @@
       <c r="N5" s="14" t="n"/>
       <c r="O5" s="14" t="inlineStr">
         <is>
-          <t>Osborne, John D</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="P5" s="14" t="n"/>
@@ -2424,7 +2424,7 @@
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
-          <t>Mosa, Abu S</t>
+          <t>Osborne, John D</t>
         </is>
       </c>
       <c r="F6" s="14" t="n"/>
@@ -2442,7 +2442,7 @@
       <c r="N6" s="14" t="n"/>
       <c r="O6" s="14" t="inlineStr">
         <is>
-          <t>Osborne, John D</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="P6" s="14" t="n"/>
@@ -2488,7 +2488,7 @@
       <c r="I7" s="14" t="n"/>
       <c r="J7" s="14" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Osborne, John D</t>
         </is>
       </c>
       <c r="K7" s="14" t="n"/>
@@ -2543,7 +2543,7 @@
       <c r="I8" s="14" t="n"/>
       <c r="J8" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="K8" s="14" t="n"/>
@@ -2552,7 +2552,7 @@
       <c r="N8" s="14" t="n"/>
       <c r="O8" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jin (Campus)</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="P8" s="14" t="n"/>
@@ -2589,7 +2589,7 @@
       </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Chong, Zechen</t>
         </is>
       </c>
       <c r="F9" s="14" t="n"/>
@@ -2598,7 +2598,7 @@
       <c r="I9" s="14" t="n"/>
       <c r="J9" s="14" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Osborne, John D</t>
         </is>
       </c>
       <c r="K9" s="14" t="n"/>
@@ -2607,7 +2607,7 @@
       <c r="N9" s="14" t="n"/>
       <c r="O9" s="14" t="inlineStr">
         <is>
-          <t>Mosa, Abu S</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="P9" s="14" t="n"/>
@@ -2644,7 +2644,7 @@
       </c>
       <c r="E10" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jin (Campus)</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="F10" s="14" t="n"/>
@@ -2653,7 +2653,7 @@
       <c r="I10" s="14" t="n"/>
       <c r="J10" s="14" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="K10" s="14" t="n"/>
@@ -2662,7 +2662,7 @@
       <c r="N10" s="14" t="n"/>
       <c r="O10" s="14" t="inlineStr">
         <is>
-          <t>Mosa, Abu S</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="P10" s="14" t="n"/>
@@ -2699,7 +2699,7 @@
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="F11" s="14" t="n"/>
@@ -2708,7 +2708,7 @@
       <c r="I11" s="14" t="n"/>
       <c r="J11" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="K11" s="14" t="n"/>
@@ -2717,7 +2717,7 @@
       <c r="N11" s="14" t="n"/>
       <c r="O11" s="14" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Chong, Zechen</t>
         </is>
       </c>
       <c r="P11" s="14" t="n"/>
@@ -2768,7 +2768,7 @@
       <c r="N12" s="14" t="n"/>
       <c r="O12" s="14" t="inlineStr">
         <is>
-          <t>Osborne, John D</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="P12" s="14" t="n"/>
@@ -2805,7 +2805,7 @@
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>Amy Wang</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="F13" s="14" t="n"/>
@@ -2814,7 +2814,7 @@
       <c r="I13" s="14" t="n"/>
       <c r="J13" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="K13" s="14" t="n"/>
@@ -2823,7 +2823,7 @@
       <c r="N13" s="14" t="n"/>
       <c r="O13" s="14" t="inlineStr">
         <is>
-          <t>Osborne, John D</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="P13" s="14" t="n"/>
@@ -2869,7 +2869,7 @@
       <c r="I14" s="14" t="n"/>
       <c r="J14" s="14" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="K14" s="14" t="n"/>
@@ -2878,7 +2878,7 @@
       <c r="N14" s="14" t="n"/>
       <c r="O14" s="14" t="inlineStr">
         <is>
-          <t>Mosa, Abu S</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="P14" s="14" t="n"/>
@@ -2915,7 +2915,7 @@
       </c>
       <c r="E15" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jin (Campus)</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="F15" s="14" t="n"/>
@@ -2933,7 +2933,7 @@
       <c r="N15" s="14" t="n"/>
       <c r="O15" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Osborne, John D</t>
         </is>
       </c>
       <c r="P15" s="14" t="n"/>
@@ -2970,7 +2970,7 @@
       </c>
       <c r="E16" s="14" t="inlineStr">
         <is>
-          <t>Amy Wang</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="F16" s="14" t="n"/>
@@ -2979,7 +2979,7 @@
       <c r="I16" s="14" t="n"/>
       <c r="J16" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Osborne, John D</t>
         </is>
       </c>
       <c r="K16" s="14" t="n"/>
@@ -2988,7 +2988,7 @@
       <c r="N16" s="14" t="n"/>
       <c r="O16" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jin (Campus)</t>
+          <t>Chong, Zechen</t>
         </is>
       </c>
       <c r="P16" s="14" t="n"/>
@@ -3025,7 +3025,7 @@
       </c>
       <c r="E17" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="F17" s="14" t="n"/>
@@ -3043,7 +3043,7 @@
       <c r="N17" s="14" t="n"/>
       <c r="O17" s="14" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Chong, Zechen</t>
         </is>
       </c>
       <c r="P17" s="14" t="n"/>
@@ -3080,7 +3080,7 @@
       </c>
       <c r="E18" s="14" t="inlineStr">
         <is>
-          <t>Amy Wang</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="F18" s="14" t="n"/>
@@ -3089,7 +3089,7 @@
       <c r="I18" s="14" t="n"/>
       <c r="J18" s="14" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="K18" s="14" t="n"/>
@@ -3135,7 +3135,7 @@
       </c>
       <c r="E19" s="14" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Chong, Zechen</t>
         </is>
       </c>
       <c r="F19" s="14" t="n"/>
@@ -3153,7 +3153,7 @@
       <c r="N19" s="14" t="n"/>
       <c r="O19" s="14" t="inlineStr">
         <is>
-          <t>Mosa, Abu S</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="P19" s="14" t="n"/>
@@ -3190,7 +3190,7 @@
       </c>
       <c r="E20" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Chong, Zechen</t>
         </is>
       </c>
       <c r="F20" s="14" t="n"/>
@@ -3199,7 +3199,7 @@
       <c r="I20" s="14" t="n"/>
       <c r="J20" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="K20" s="14" t="n"/>
@@ -3208,7 +3208,7 @@
       <c r="N20" s="14" t="n"/>
       <c r="O20" s="14" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="P20" s="14" t="n"/>
@@ -3254,7 +3254,7 @@
       <c r="I21" s="14" t="n"/>
       <c r="J21" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Osborne, John D</t>
         </is>
       </c>
       <c r="K21" s="14" t="n"/>
@@ -3263,7 +3263,7 @@
       <c r="N21" s="14" t="n"/>
       <c r="O21" s="14" t="inlineStr">
         <is>
-          <t>Osborne, John D</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="P21" s="14" t="n"/>
@@ -3300,7 +3300,7 @@
       </c>
       <c r="E22" s="14" t="inlineStr">
         <is>
-          <t>Amy Wang</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="F22" s="14" t="n"/>
@@ -3309,7 +3309,7 @@
       <c r="I22" s="14" t="n"/>
       <c r="J22" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="K22" s="14" t="n"/>
@@ -3364,7 +3364,7 @@
       <c r="I23" s="14" t="n"/>
       <c r="J23" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jin (Campus)</t>
+          <t>Chong, Zechen</t>
         </is>
       </c>
       <c r="K23" s="14" t="n"/>
@@ -3373,7 +3373,7 @@
       <c r="N23" s="14" t="n"/>
       <c r="O23" s="14" t="inlineStr">
         <is>
-          <t>Mosa, Abu S</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="P23" s="14" t="n"/>
@@ -3419,7 +3419,7 @@
       <c r="I24" s="14" t="n"/>
       <c r="J24" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Osborne, John D</t>
         </is>
       </c>
       <c r="K24" s="14" t="n"/>
@@ -3428,7 +3428,7 @@
       <c r="N24" s="14" t="n"/>
       <c r="O24" s="14" t="inlineStr">
         <is>
-          <t>Osborne, John D</t>
+          <t>Chong, Zechen</t>
         </is>
       </c>
       <c r="P24" s="14" t="n"/>
@@ -3465,7 +3465,7 @@
       </c>
       <c r="E25" s="14" t="inlineStr">
         <is>
-          <t>Chong, Zechen</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="F25" s="14" t="n"/>
@@ -3474,7 +3474,7 @@
       <c r="I25" s="14" t="n"/>
       <c r="J25" s="14" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="K25" s="14" t="n"/>
@@ -3483,7 +3483,7 @@
       <c r="N25" s="14" t="n"/>
       <c r="O25" s="14" t="inlineStr">
         <is>
-          <t>Mosa, Abu S</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="P25" s="14" t="n"/>
@@ -3529,7 +3529,7 @@
       <c r="I26" s="14" t="n"/>
       <c r="J26" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jin (Campus)</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="K26" s="14" t="n"/>
@@ -3538,7 +3538,7 @@
       <c r="N26" s="14" t="n"/>
       <c r="O26" s="14" t="inlineStr">
         <is>
-          <t>Mosa, Abu S</t>
+          <t>Amy Wang</t>
         </is>
       </c>
       <c r="P26" s="14" t="n"/>
@@ -3584,7 +3584,7 @@
       <c r="I27" s="14" t="n"/>
       <c r="J27" s="14" t="inlineStr">
         <is>
-          <t>Amy Wang</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="K27" s="14" t="n"/>
@@ -3593,7 +3593,7 @@
       <c r="N27" s="14" t="n"/>
       <c r="O27" s="14" t="inlineStr">
         <is>
-          <t>Osborne, John D</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="P27" s="14" t="n"/>
@@ -3639,7 +3639,7 @@
       <c r="I28" s="14" t="n"/>
       <c r="J28" s="14" t="inlineStr">
         <is>
-          <t>Amy Wang</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="K28" s="14" t="n"/>
@@ -3648,7 +3648,7 @@
       <c r="N28" s="14" t="n"/>
       <c r="O28" s="14" t="inlineStr">
         <is>
-          <t>Osborne, John D</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="P28" s="14" t="n"/>
@@ -3694,7 +3694,7 @@
       <c r="I29" s="14" t="n"/>
       <c r="J29" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="K29" s="14" t="n"/>
@@ -3703,7 +3703,7 @@
       <c r="N29" s="14" t="n"/>
       <c r="O29" s="14" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="P29" s="14" t="n"/>
@@ -3740,7 +3740,7 @@
       </c>
       <c r="E30" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Chen, Jin (Campus)</t>
         </is>
       </c>
       <c r="F30" s="14" t="n"/>
@@ -3749,7 +3749,7 @@
       <c r="I30" s="14" t="n"/>
       <c r="J30" s="14" t="inlineStr">
         <is>
-          <t>Chen, Jin (Campus)</t>
+          <t>Mosa, Abu S</t>
         </is>
       </c>
       <c r="K30" s="14" t="n"/>
@@ -3758,7 +3758,7 @@
       <c r="N30" s="14" t="n"/>
       <c r="O30" s="14" t="inlineStr">
         <is>
-          <t>Mosa, Abu S</t>
+          <t>Chen, Jake Y</t>
         </is>
       </c>
       <c r="P30" s="14" t="n"/>
@@ -3802,12 +3802,12 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Chen, Jake Y</t>
+          <t>Jinzhuang Dou</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>Jinzhuang Dou</t>
+          <t>Chong, Zechen</t>
         </is>
       </c>
     </row>

</xml_diff>